<commit_message>
Updated Excel after final corrections
</commit_message>
<xml_diff>
--- a/IT23681842-Assignment 1 - Test cases.xlsx
+++ b/IT23681842-Assignment 1 - Test cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SLIIT\3rd Year\1st Semester\ITPM\ITPM Assignment IT23681842\test_automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SLIIT\3rd Year\1st Semester\ITPM\ITPM Assignment IT23681842\IT23681842\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA449D70-C38F-42A0-BA0A-8B07E2FA86CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46FE1579-FD1D-4722-87FE-8B1C00FB262D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="292">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -899,6 +899,9 @@
   </si>
   <si>
     <t>Includes “Tiranya Fashion,” English words, and emoji.</t>
+  </si>
+  <si>
+    <t>S</t>
   </si>
 </sst>
 </file>
@@ -1009,25 +1012,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1348,2777 +1351,2875 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="9" t="s">
+      <c r="F2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="2" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="B6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" s="9" t="s">
+      <c r="F6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="2" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="9" t="s">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="2" t="s">
         <v>212</v>
       </c>
       <c r="H7" s="1"/>
     </row>
     <row r="8" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="B10" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="F10" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="9" t="s">
+      <c r="F10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="2" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="9" t="s">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="2" t="s">
         <v>215</v>
       </c>
       <c r="H11" s="1"/>
     </row>
     <row r="12" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
     </row>
     <row r="13" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
     </row>
     <row r="14" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="2" t="s">
+      <c r="B14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" s="9" t="s">
+      <c r="F14" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H14" s="2" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="9" t="s">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="2" t="s">
         <v>215</v>
       </c>
       <c r="H15" s="1"/>
     </row>
     <row r="16" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
     </row>
     <row r="17" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
     </row>
     <row r="18" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="2" t="s">
+      <c r="B18" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G18" s="9" t="s">
+      <c r="F18" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="H18" s="2" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="9" t="s">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="2" t="s">
         <v>220</v>
       </c>
       <c r="H19" s="1"/>
     </row>
     <row r="20" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
     </row>
     <row r="21" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
     </row>
     <row r="22" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="2" t="s">
+      <c r="B22" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G22" s="9" t="s">
+      <c r="F22" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="H22" s="2" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
     </row>
     <row r="24" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
     </row>
     <row r="25" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
     </row>
     <row r="26" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="7"/>
-      <c r="C26" s="2" t="s">
+      <c r="B26" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="F26" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G26" s="9" t="s">
+      <c r="F26" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="2" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="9" t="s">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="2" t="s">
         <v>212</v>
       </c>
       <c r="H27" s="1"/>
     </row>
     <row r="28" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="9"/>
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="2"/>
       <c r="H28" s="1"/>
     </row>
     <row r="29" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
     </row>
     <row r="30" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="8" t="s">
+      <c r="A30" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="7"/>
-      <c r="C30" s="2" t="s">
+      <c r="B30" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="E30" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F30" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" s="9" t="s">
+      <c r="F30" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="H30" s="9" t="s">
+      <c r="H30" s="2" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="9" t="s">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="2" t="s">
         <v>212</v>
       </c>
       <c r="H31" s="1"/>
     </row>
     <row r="32" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
     </row>
     <row r="33" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
+      <c r="A33" s="5"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
     </row>
     <row r="34" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="7"/>
-      <c r="C34" s="2" t="s">
+      <c r="B34" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="D34" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="E34" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F34" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34" s="9" t="s">
+      <c r="F34" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H34" s="2" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="9" t="s">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="2" t="s">
         <v>225</v>
       </c>
       <c r="H35" s="1"/>
     </row>
     <row r="36" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
     </row>
     <row r="37" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
+      <c r="A37" s="5"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
     </row>
     <row r="38" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="7"/>
-      <c r="C38" s="2" t="s">
+      <c r="B38" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D38" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E38" s="5" t="s">
+      <c r="E38" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="F38" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G38" s="9" t="s">
+      <c r="F38" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="H38" s="9" t="s">
+      <c r="H38" s="2" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
     </row>
     <row r="40" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
-      <c r="F40" s="3"/>
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
     </row>
     <row r="41" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="4"/>
-      <c r="B41" s="4"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
     </row>
     <row r="42" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="8" t="s">
+      <c r="A42" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B42" s="7"/>
-      <c r="C42" s="2" t="s">
+      <c r="B42" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D42" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="E42" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="F42" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G42" s="9" t="s">
+      <c r="F42" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="H42" s="2" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-      <c r="F43" s="3"/>
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
     </row>
     <row r="44" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
-      <c r="F44" s="3"/>
+      <c r="A44" s="4"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
     </row>
     <row r="45" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
     </row>
     <row r="46" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="8" t="s">
+      <c r="A46" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B46" s="7"/>
-      <c r="C46" s="2" t="s">
+      <c r="B46" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C46" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="D46" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="E46" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="F46" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G46" s="9" t="s">
+      <c r="F46" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G46" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="H46" s="9" t="s">
+      <c r="H46" s="2" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
+      <c r="A47" s="4"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
     </row>
     <row r="48" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
     </row>
     <row r="49" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="4"/>
-      <c r="B49" s="4"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
+      <c r="A49" s="5"/>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
     </row>
     <row r="50" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="8" t="s">
+      <c r="A50" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B50" s="7"/>
-      <c r="C50" s="2" t="s">
+      <c r="B50" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C50" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="D50" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E50" s="5" t="s">
+      <c r="E50" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="F50" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G50" s="9" t="s">
+      <c r="F50" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G50" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="H50" s="9" t="s">
+      <c r="H50" s="2" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
-      <c r="G51" s="9" t="s">
+      <c r="A51" s="4"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="2" t="s">
         <v>233</v>
       </c>
       <c r="H51" s="1"/>
     </row>
     <row r="52" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
+      <c r="A52" s="4"/>
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
     </row>
     <row r="53" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="4"/>
-      <c r="B53" s="4"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
+      <c r="A53" s="5"/>
+      <c r="B53" s="5"/>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
     </row>
     <row r="54" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="8" t="s">
+      <c r="A54" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B54" s="7"/>
-      <c r="C54" s="2" t="s">
+      <c r="B54" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D54" s="6" t="s">
+      <c r="D54" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E54" s="5" t="s">
+      <c r="E54" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="F54" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G54" s="9" t="s">
+      <c r="F54" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G54" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H54" s="9" t="s">
+      <c r="H54" s="2" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="3"/>
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
-      <c r="F55" s="3"/>
+      <c r="A55" s="4"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
     </row>
     <row r="56" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="3"/>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
-      <c r="E56" s="3"/>
-      <c r="F56" s="3"/>
+      <c r="A56" s="4"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
     </row>
     <row r="57" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="4"/>
-      <c r="B57" s="4"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
+      <c r="A57" s="5"/>
+      <c r="B57" s="5"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
     </row>
     <row r="58" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="8" t="s">
+      <c r="A58" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B58" s="7"/>
-      <c r="C58" s="2" t="s">
+      <c r="B58" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C58" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D58" s="6" t="s">
+      <c r="D58" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E58" s="5" t="s">
+      <c r="E58" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="F58" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G58" s="9" t="s">
+      <c r="F58" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G58" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="H58" s="9" t="s">
+      <c r="H58" s="2" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="3"/>
-      <c r="B59" s="3"/>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
-      <c r="F59" s="3"/>
-      <c r="G59" s="9" t="s">
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="2" t="s">
         <v>217</v>
       </c>
       <c r="H59" s="1"/>
     </row>
     <row r="60" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="3"/>
-      <c r="B60" s="3"/>
-      <c r="C60" s="3"/>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
-      <c r="F60" s="3"/>
+      <c r="A60" s="4"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>
     </row>
     <row r="61" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
-      <c r="F61" s="4"/>
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
       <c r="G61" s="1"/>
       <c r="H61" s="1"/>
     </row>
     <row r="62" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="8" t="s">
+      <c r="A62" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B62" s="7"/>
-      <c r="C62" s="2" t="s">
+      <c r="B62" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D62" s="6" t="s">
+      <c r="D62" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E62" s="5" t="s">
+      <c r="E62" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="F62" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G62" s="9" t="s">
+      <c r="F62" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G62" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H62" s="9" t="s">
+      <c r="H62" s="2" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="3"/>
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="3"/>
-      <c r="E63" s="3"/>
-      <c r="F63" s="3"/>
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4"/>
       <c r="G63" s="1"/>
       <c r="H63" s="1"/>
     </row>
     <row r="64" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
-      <c r="E64" s="3"/>
-      <c r="F64" s="3"/>
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
     </row>
     <row r="65" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="4"/>
-      <c r="B65" s="4"/>
-      <c r="C65" s="4"/>
-      <c r="D65" s="4"/>
-      <c r="E65" s="4"/>
-      <c r="F65" s="4"/>
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
+      <c r="C65" s="5"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
     </row>
     <row r="66" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="8" t="s">
+      <c r="A66" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B66" s="7"/>
-      <c r="C66" s="2" t="s">
+      <c r="B66" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C66" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D66" s="6" t="s">
+      <c r="D66" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E66" s="5" t="s">
+      <c r="E66" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="F66" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G66" s="9" t="s">
+      <c r="F66" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G66" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="H66" s="9" t="s">
+      <c r="H66" s="2" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="3"/>
-      <c r="B67" s="3"/>
-      <c r="C67" s="3"/>
-      <c r="D67" s="3"/>
-      <c r="E67" s="3"/>
-      <c r="F67" s="3"/>
-      <c r="G67" s="9" t="s">
+      <c r="A67" s="4"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4"/>
+      <c r="G67" s="2" t="s">
         <v>240</v>
       </c>
       <c r="H67" s="1"/>
     </row>
     <row r="68" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="3"/>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
+      <c r="A68" s="4"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="4"/>
+      <c r="F68" s="4"/>
       <c r="G68" s="1"/>
       <c r="H68" s="1"/>
     </row>
     <row r="69" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="4"/>
-      <c r="B69" s="4"/>
-      <c r="C69" s="4"/>
-      <c r="D69" s="4"/>
-      <c r="E69" s="4"/>
-      <c r="F69" s="4"/>
+      <c r="A69" s="5"/>
+      <c r="B69" s="5"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
       <c r="G69" s="1"/>
       <c r="H69" s="1"/>
     </row>
     <row r="70" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="8" t="s">
+      <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B70" s="7"/>
-      <c r="C70" s="2" t="s">
+      <c r="B70" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C70" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="D70" s="6" t="s">
+      <c r="D70" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E70" s="5" t="s">
+      <c r="E70" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="F70" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G70" s="9" t="s">
+      <c r="F70" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G70" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="H70" s="9" t="s">
+      <c r="H70" s="2" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="3"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="3"/>
-      <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
+      <c r="A71" s="4"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
       <c r="G71" s="1"/>
       <c r="H71" s="1"/>
     </row>
     <row r="72" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="3"/>
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
+      <c r="A72" s="4"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4"/>
       <c r="G72" s="1"/>
       <c r="H72" s="1"/>
     </row>
     <row r="73" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="4"/>
-      <c r="B73" s="4"/>
-      <c r="C73" s="4"/>
-      <c r="D73" s="4"/>
-      <c r="E73" s="4"/>
-      <c r="F73" s="4"/>
+      <c r="A73" s="5"/>
+      <c r="B73" s="5"/>
+      <c r="C73" s="5"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
       <c r="G73" s="1"/>
       <c r="H73" s="1"/>
     </row>
     <row r="74" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="8" t="s">
+      <c r="A74" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B74" s="7"/>
-      <c r="C74" s="2" t="s">
+      <c r="B74" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C74" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="D74" s="6" t="s">
+      <c r="D74" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="E74" s="5" t="s">
+      <c r="E74" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="F74" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G74" s="9" t="s">
+      <c r="F74" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G74" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="H74" s="9" t="s">
+      <c r="H74" s="2" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="3"/>
-      <c r="B75" s="3"/>
-      <c r="C75" s="3"/>
-      <c r="D75" s="3"/>
-      <c r="E75" s="3"/>
-      <c r="F75" s="3"/>
+      <c r="A75" s="4"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
       <c r="G75" s="1"/>
       <c r="H75" s="1"/>
     </row>
     <row r="76" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="3"/>
-      <c r="B76" s="3"/>
-      <c r="C76" s="3"/>
-      <c r="D76" s="3"/>
-      <c r="E76" s="3"/>
-      <c r="F76" s="3"/>
+      <c r="A76" s="4"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="4"/>
+      <c r="E76" s="4"/>
+      <c r="F76" s="4"/>
       <c r="G76" s="1"/>
       <c r="H76" s="1"/>
     </row>
     <row r="77" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="4"/>
-      <c r="B77" s="4"/>
-      <c r="C77" s="4"/>
-      <c r="D77" s="4"/>
-      <c r="E77" s="4"/>
-      <c r="F77" s="4"/>
+      <c r="A77" s="5"/>
+      <c r="B77" s="5"/>
+      <c r="C77" s="5"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
       <c r="G77" s="1"/>
       <c r="H77" s="1"/>
     </row>
     <row r="78" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="8" t="s">
+      <c r="A78" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B78" s="7"/>
-      <c r="C78" s="2" t="s">
+      <c r="B78" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C78" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D78" s="6" t="s">
+      <c r="D78" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E78" s="5" t="s">
+      <c r="E78" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="F78" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G78" s="9" t="s">
+      <c r="F78" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G78" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="H78" s="9" t="s">
+      <c r="H78" s="2" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="3"/>
-      <c r="B79" s="3"/>
-      <c r="C79" s="3"/>
-      <c r="D79" s="3"/>
-      <c r="E79" s="3"/>
-      <c r="F79" s="3"/>
+      <c r="A79" s="4"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4"/>
+      <c r="F79" s="4"/>
       <c r="G79" s="1"/>
       <c r="H79" s="1"/>
     </row>
     <row r="80" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="3"/>
-      <c r="B80" s="3"/>
-      <c r="C80" s="3"/>
-      <c r="D80" s="3"/>
-      <c r="E80" s="3"/>
-      <c r="F80" s="3"/>
+      <c r="A80" s="4"/>
+      <c r="B80" s="4"/>
+      <c r="C80" s="4"/>
+      <c r="D80" s="4"/>
+      <c r="E80" s="4"/>
+      <c r="F80" s="4"/>
       <c r="G80" s="1"/>
       <c r="H80" s="1"/>
     </row>
     <row r="81" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="4"/>
-      <c r="B81" s="4"/>
-      <c r="C81" s="4"/>
-      <c r="D81" s="4"/>
-      <c r="E81" s="4"/>
-      <c r="F81" s="4"/>
+      <c r="A81" s="5"/>
+      <c r="B81" s="5"/>
+      <c r="C81" s="5"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
       <c r="G81" s="1"/>
       <c r="H81" s="1"/>
     </row>
     <row r="82" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="8" t="s">
+      <c r="A82" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B82" s="7"/>
-      <c r="C82" s="2" t="s">
+      <c r="B82" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C82" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="D82" s="6" t="s">
+      <c r="D82" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E82" s="5" t="s">
+      <c r="E82" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="F82" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G82" s="9" t="s">
+      <c r="F82" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G82" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="H82" s="9" t="s">
+      <c r="H82" s="2" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="3"/>
-      <c r="B83" s="3"/>
-      <c r="C83" s="3"/>
-      <c r="D83" s="3"/>
-      <c r="E83" s="3"/>
-      <c r="F83" s="3"/>
+      <c r="A83" s="4"/>
+      <c r="B83" s="4"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
       <c r="G83" s="1"/>
       <c r="H83" s="1"/>
     </row>
     <row r="84" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="3"/>
-      <c r="B84" s="3"/>
-      <c r="C84" s="3"/>
-      <c r="D84" s="3"/>
-      <c r="E84" s="3"/>
-      <c r="F84" s="3"/>
+      <c r="A84" s="4"/>
+      <c r="B84" s="4"/>
+      <c r="C84" s="4"/>
+      <c r="D84" s="4"/>
+      <c r="E84" s="4"/>
+      <c r="F84" s="4"/>
       <c r="G84" s="1"/>
       <c r="H84" s="1"/>
     </row>
     <row r="85" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="4"/>
-      <c r="B85" s="4"/>
-      <c r="C85" s="4"/>
-      <c r="D85" s="4"/>
-      <c r="E85" s="4"/>
-      <c r="F85" s="4"/>
+      <c r="A85" s="5"/>
+      <c r="B85" s="5"/>
+      <c r="C85" s="5"/>
+      <c r="D85" s="5"/>
+      <c r="E85" s="5"/>
+      <c r="F85" s="5"/>
       <c r="G85" s="1"/>
       <c r="H85" s="1"/>
     </row>
     <row r="86" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="8" t="s">
+      <c r="A86" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B86" s="7"/>
-      <c r="C86" s="2" t="s">
+      <c r="B86" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C86" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="D86" s="6" t="s">
+      <c r="D86" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E86" s="5" t="s">
+      <c r="E86" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="F86" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G86" s="9" t="s">
+      <c r="F86" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G86" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="H86" s="9" t="s">
+      <c r="H86" s="2" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="3"/>
-      <c r="B87" s="3"/>
-      <c r="C87" s="3"/>
-      <c r="D87" s="3"/>
-      <c r="E87" s="3"/>
-      <c r="F87" s="3"/>
+      <c r="A87" s="4"/>
+      <c r="B87" s="4"/>
+      <c r="C87" s="4"/>
+      <c r="D87" s="4"/>
+      <c r="E87" s="4"/>
+      <c r="F87" s="4"/>
       <c r="G87" s="1"/>
       <c r="H87" s="1"/>
     </row>
     <row r="88" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="3"/>
-      <c r="B88" s="3"/>
-      <c r="C88" s="3"/>
-      <c r="D88" s="3"/>
-      <c r="E88" s="3"/>
-      <c r="F88" s="3"/>
+      <c r="A88" s="4"/>
+      <c r="B88" s="4"/>
+      <c r="C88" s="4"/>
+      <c r="D88" s="4"/>
+      <c r="E88" s="4"/>
+      <c r="F88" s="4"/>
       <c r="G88" s="1"/>
       <c r="H88" s="1"/>
     </row>
     <row r="89" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="4"/>
-      <c r="B89" s="4"/>
-      <c r="C89" s="4"/>
-      <c r="D89" s="4"/>
-      <c r="E89" s="4"/>
-      <c r="F89" s="4"/>
+      <c r="A89" s="5"/>
+      <c r="B89" s="5"/>
+      <c r="C89" s="5"/>
+      <c r="D89" s="5"/>
+      <c r="E89" s="5"/>
+      <c r="F89" s="5"/>
       <c r="G89" s="1"/>
       <c r="H89" s="1"/>
     </row>
     <row r="90" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="8" t="s">
+      <c r="A90" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B90" s="7"/>
-      <c r="C90" s="2" t="s">
+      <c r="B90" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C90" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D90" s="6" t="s">
+      <c r="D90" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="E90" s="5" t="s">
+      <c r="E90" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="F90" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G90" s="9" t="s">
+      <c r="F90" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G90" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="H90" s="9" t="s">
+      <c r="H90" s="2" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="3"/>
-      <c r="B91" s="3"/>
-      <c r="C91" s="3"/>
-      <c r="D91" s="3"/>
-      <c r="E91" s="3"/>
-      <c r="F91" s="3"/>
+      <c r="A91" s="4"/>
+      <c r="B91" s="4"/>
+      <c r="C91" s="4"/>
+      <c r="D91" s="4"/>
+      <c r="E91" s="4"/>
+      <c r="F91" s="4"/>
       <c r="G91" s="1"/>
       <c r="H91" s="1"/>
     </row>
     <row r="92" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="3"/>
-      <c r="B92" s="3"/>
-      <c r="C92" s="3"/>
-      <c r="D92" s="3"/>
-      <c r="E92" s="3"/>
-      <c r="F92" s="3"/>
+      <c r="A92" s="4"/>
+      <c r="B92" s="4"/>
+      <c r="C92" s="4"/>
+      <c r="D92" s="4"/>
+      <c r="E92" s="4"/>
+      <c r="F92" s="4"/>
       <c r="G92" s="1"/>
       <c r="H92" s="1"/>
     </row>
     <row r="93" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="4"/>
-      <c r="B93" s="4"/>
-      <c r="C93" s="4"/>
-      <c r="D93" s="4"/>
-      <c r="E93" s="4"/>
-      <c r="F93" s="4"/>
+      <c r="A93" s="5"/>
+      <c r="B93" s="5"/>
+      <c r="C93" s="5"/>
+      <c r="D93" s="5"/>
+      <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
       <c r="G93" s="1"/>
       <c r="H93" s="1"/>
     </row>
     <row r="94" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="8" t="s">
+      <c r="A94" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B94" s="7"/>
-      <c r="C94" s="2" t="s">
+      <c r="B94" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C94" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D94" s="6" t="s">
+      <c r="D94" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E94" s="5" t="s">
+      <c r="E94" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="F94" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G94" s="9" t="s">
+      <c r="F94" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G94" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="H94" s="9" t="s">
+      <c r="H94" s="2" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="3"/>
-      <c r="B95" s="3"/>
-      <c r="C95" s="3"/>
-      <c r="D95" s="3"/>
-      <c r="E95" s="3"/>
-      <c r="F95" s="3"/>
+      <c r="A95" s="4"/>
+      <c r="B95" s="4"/>
+      <c r="C95" s="4"/>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+      <c r="F95" s="4"/>
       <c r="G95" s="1"/>
       <c r="H95" s="1"/>
     </row>
     <row r="96" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="3"/>
-      <c r="B96" s="3"/>
-      <c r="C96" s="3"/>
-      <c r="D96" s="3"/>
-      <c r="E96" s="3"/>
-      <c r="F96" s="3"/>
+      <c r="A96" s="4"/>
+      <c r="B96" s="4"/>
+      <c r="C96" s="4"/>
+      <c r="D96" s="4"/>
+      <c r="E96" s="4"/>
+      <c r="F96" s="4"/>
       <c r="G96" s="1"/>
       <c r="H96" s="1"/>
     </row>
     <row r="97" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="4"/>
-      <c r="B97" s="4"/>
-      <c r="C97" s="4"/>
-      <c r="D97" s="4"/>
-      <c r="E97" s="4"/>
-      <c r="F97" s="4"/>
+      <c r="A97" s="5"/>
+      <c r="B97" s="5"/>
+      <c r="C97" s="5"/>
+      <c r="D97" s="5"/>
+      <c r="E97" s="5"/>
+      <c r="F97" s="5"/>
       <c r="G97" s="1"/>
       <c r="H97" s="1"/>
     </row>
     <row r="98" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="8" t="s">
+      <c r="A98" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B98" s="7"/>
-      <c r="C98" s="2" t="s">
+      <c r="B98" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C98" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="D98" s="6" t="s">
+      <c r="D98" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E98" s="5" t="s">
+      <c r="E98" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="F98" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G98" s="9" t="s">
+      <c r="F98" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G98" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="H98" s="9" t="s">
+      <c r="H98" s="2" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="3"/>
-      <c r="B99" s="3"/>
-      <c r="C99" s="3"/>
-      <c r="D99" s="3"/>
-      <c r="E99" s="3"/>
-      <c r="F99" s="3"/>
+      <c r="A99" s="4"/>
+      <c r="B99" s="4"/>
+      <c r="C99" s="4"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
       <c r="G99" s="1"/>
       <c r="H99" s="1"/>
     </row>
     <row r="100" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="3"/>
-      <c r="B100" s="3"/>
-      <c r="C100" s="3"/>
-      <c r="D100" s="3"/>
-      <c r="E100" s="3"/>
-      <c r="F100" s="3"/>
+      <c r="A100" s="4"/>
+      <c r="B100" s="4"/>
+      <c r="C100" s="4"/>
+      <c r="D100" s="4"/>
+      <c r="E100" s="4"/>
+      <c r="F100" s="4"/>
       <c r="G100" s="1"/>
       <c r="H100" s="1"/>
     </row>
     <row r="101" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="4"/>
-      <c r="B101" s="4"/>
-      <c r="C101" s="4"/>
-      <c r="D101" s="4"/>
-      <c r="E101" s="4"/>
-      <c r="F101" s="4"/>
+      <c r="A101" s="5"/>
+      <c r="B101" s="5"/>
+      <c r="C101" s="5"/>
+      <c r="D101" s="5"/>
+      <c r="E101" s="5"/>
+      <c r="F101" s="5"/>
       <c r="G101" s="1"/>
       <c r="H101" s="1"/>
     </row>
     <row r="102" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="8" t="s">
+      <c r="A102" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B102" s="7"/>
-      <c r="C102" s="2" t="s">
+      <c r="B102" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C102" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="D102" s="6" t="s">
+      <c r="D102" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E102" s="5" t="s">
+      <c r="E102" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="F102" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G102" s="9" t="s">
+      <c r="F102" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G102" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="H102" s="9" t="s">
+      <c r="H102" s="2" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="3"/>
-      <c r="B103" s="3"/>
-      <c r="C103" s="3"/>
-      <c r="D103" s="3"/>
-      <c r="E103" s="3"/>
-      <c r="F103" s="3"/>
-      <c r="G103" s="9" t="s">
+      <c r="A103" s="4"/>
+      <c r="B103" s="4"/>
+      <c r="C103" s="4"/>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4"/>
+      <c r="G103" s="2" t="s">
         <v>254</v>
       </c>
       <c r="H103" s="1"/>
     </row>
     <row r="104" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="3"/>
-      <c r="B104" s="3"/>
-      <c r="C104" s="3"/>
-      <c r="D104" s="3"/>
-      <c r="E104" s="3"/>
-      <c r="F104" s="3"/>
+      <c r="A104" s="4"/>
+      <c r="B104" s="4"/>
+      <c r="C104" s="4"/>
+      <c r="D104" s="4"/>
+      <c r="E104" s="4"/>
+      <c r="F104" s="4"/>
       <c r="G104" s="1"/>
       <c r="H104" s="1"/>
     </row>
     <row r="105" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="4"/>
-      <c r="B105" s="4"/>
-      <c r="C105" s="4"/>
-      <c r="D105" s="4"/>
-      <c r="E105" s="4"/>
-      <c r="F105" s="4"/>
+      <c r="A105" s="5"/>
+      <c r="B105" s="5"/>
+      <c r="C105" s="5"/>
+      <c r="D105" s="5"/>
+      <c r="E105" s="5"/>
+      <c r="F105" s="5"/>
       <c r="G105" s="1"/>
       <c r="H105" s="1"/>
     </row>
     <row r="106" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="8" t="s">
+      <c r="A106" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B106" s="7"/>
-      <c r="C106" s="2" t="s">
+      <c r="B106" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C106" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="D106" s="6" t="s">
+      <c r="D106" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="E106" s="5" t="s">
+      <c r="E106" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="F106" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G106" s="9" t="s">
+      <c r="F106" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G106" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="H106" s="9" t="s">
+      <c r="H106" s="2" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="107" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="3"/>
-      <c r="B107" s="3"/>
-      <c r="C107" s="3"/>
-      <c r="D107" s="3"/>
-      <c r="E107" s="3"/>
-      <c r="F107" s="3"/>
-      <c r="G107" s="9" t="s">
+      <c r="A107" s="4"/>
+      <c r="B107" s="4"/>
+      <c r="C107" s="4"/>
+      <c r="D107" s="4"/>
+      <c r="E107" s="4"/>
+      <c r="F107" s="4"/>
+      <c r="G107" s="2" t="s">
         <v>256</v>
       </c>
       <c r="H107" s="1"/>
     </row>
     <row r="108" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="3"/>
-      <c r="B108" s="3"/>
-      <c r="C108" s="3"/>
-      <c r="D108" s="3"/>
-      <c r="E108" s="3"/>
-      <c r="F108" s="3"/>
+      <c r="A108" s="4"/>
+      <c r="B108" s="4"/>
+      <c r="C108" s="4"/>
+      <c r="D108" s="4"/>
+      <c r="E108" s="4"/>
+      <c r="F108" s="4"/>
       <c r="G108" s="1"/>
       <c r="H108" s="1"/>
     </row>
     <row r="109" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="4"/>
-      <c r="B109" s="4"/>
-      <c r="C109" s="4"/>
-      <c r="D109" s="4"/>
-      <c r="E109" s="4"/>
-      <c r="F109" s="4"/>
+      <c r="A109" s="5"/>
+      <c r="B109" s="5"/>
+      <c r="C109" s="5"/>
+      <c r="D109" s="5"/>
+      <c r="E109" s="5"/>
+      <c r="F109" s="5"/>
       <c r="G109" s="1"/>
       <c r="H109" s="1"/>
     </row>
     <row r="110" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="8" t="s">
+      <c r="A110" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B110" s="7"/>
-      <c r="C110" s="2" t="s">
+      <c r="B110" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C110" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="D110" s="6" t="s">
+      <c r="D110" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E110" s="5" t="s">
+      <c r="E110" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="F110" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G110" s="9" t="s">
+      <c r="F110" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G110" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="H110" s="9" t="s">
+      <c r="H110" s="2" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="3"/>
-      <c r="B111" s="3"/>
-      <c r="C111" s="3"/>
-      <c r="D111" s="3"/>
-      <c r="E111" s="3"/>
-      <c r="F111" s="3"/>
+      <c r="A111" s="4"/>
+      <c r="B111" s="4"/>
+      <c r="C111" s="4"/>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
       <c r="G111" s="1"/>
       <c r="H111" s="1"/>
     </row>
     <row r="112" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A112" s="3"/>
-      <c r="B112" s="3"/>
-      <c r="C112" s="3"/>
-      <c r="D112" s="3"/>
-      <c r="E112" s="3"/>
-      <c r="F112" s="3"/>
+      <c r="A112" s="4"/>
+      <c r="B112" s="4"/>
+      <c r="C112" s="4"/>
+      <c r="D112" s="4"/>
+      <c r="E112" s="4"/>
+      <c r="F112" s="4"/>
       <c r="G112" s="1"/>
       <c r="H112" s="1"/>
     </row>
     <row r="113" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="4"/>
-      <c r="B113" s="4"/>
-      <c r="C113" s="4"/>
-      <c r="D113" s="4"/>
-      <c r="E113" s="4"/>
-      <c r="F113" s="4"/>
+      <c r="A113" s="5"/>
+      <c r="B113" s="5"/>
+      <c r="C113" s="5"/>
+      <c r="D113" s="5"/>
+      <c r="E113" s="5"/>
+      <c r="F113" s="5"/>
       <c r="G113" s="1"/>
       <c r="H113" s="1"/>
     </row>
     <row r="114" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="8" t="s">
+      <c r="A114" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B114" s="7"/>
-      <c r="C114" s="2" t="s">
+      <c r="B114" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C114" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D114" s="6" t="s">
+      <c r="D114" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E114" s="5" t="s">
+      <c r="E114" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="F114" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G114" s="9" t="s">
+      <c r="F114" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G114" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="H114" s="9" t="s">
+      <c r="H114" s="2" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="3"/>
-      <c r="B115" s="3"/>
-      <c r="C115" s="3"/>
-      <c r="D115" s="3"/>
-      <c r="E115" s="3"/>
-      <c r="F115" s="3"/>
-      <c r="G115" s="9" t="s">
+      <c r="A115" s="4"/>
+      <c r="B115" s="4"/>
+      <c r="C115" s="4"/>
+      <c r="D115" s="4"/>
+      <c r="E115" s="4"/>
+      <c r="F115" s="4"/>
+      <c r="G115" s="2" t="s">
         <v>256</v>
       </c>
       <c r="H115" s="1"/>
     </row>
     <row r="116" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="3"/>
-      <c r="B116" s="3"/>
-      <c r="C116" s="3"/>
-      <c r="D116" s="3"/>
-      <c r="E116" s="3"/>
-      <c r="F116" s="3"/>
+      <c r="A116" s="4"/>
+      <c r="B116" s="4"/>
+      <c r="C116" s="4"/>
+      <c r="D116" s="4"/>
+      <c r="E116" s="4"/>
+      <c r="F116" s="4"/>
       <c r="G116" s="1"/>
       <c r="H116" s="1"/>
     </row>
     <row r="117" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="4"/>
-      <c r="B117" s="4"/>
-      <c r="C117" s="4"/>
-      <c r="D117" s="4"/>
-      <c r="E117" s="4"/>
-      <c r="F117" s="4"/>
+      <c r="A117" s="5"/>
+      <c r="B117" s="5"/>
+      <c r="C117" s="5"/>
+      <c r="D117" s="5"/>
+      <c r="E117" s="5"/>
+      <c r="F117" s="5"/>
       <c r="G117" s="1"/>
       <c r="H117" s="1"/>
     </row>
     <row r="118" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A118" s="8" t="s">
+      <c r="A118" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B118" s="7"/>
-      <c r="C118" s="2" t="s">
+      <c r="B118" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C118" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="D118" s="6" t="s">
+      <c r="D118" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E118" s="5" t="s">
+      <c r="E118" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="F118" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G118" s="9" t="s">
+      <c r="F118" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G118" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="H118" s="9" t="s">
+      <c r="H118" s="2" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="3"/>
-      <c r="B119" s="3"/>
-      <c r="C119" s="3"/>
-      <c r="D119" s="3"/>
-      <c r="E119" s="3"/>
-      <c r="F119" s="3"/>
-      <c r="G119" s="9" t="s">
+      <c r="A119" s="4"/>
+      <c r="B119" s="4"/>
+      <c r="C119" s="4"/>
+      <c r="D119" s="4"/>
+      <c r="E119" s="4"/>
+      <c r="F119" s="4"/>
+      <c r="G119" s="2" t="s">
         <v>210</v>
       </c>
       <c r="H119" s="1"/>
     </row>
     <row r="120" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="3"/>
-      <c r="B120" s="3"/>
-      <c r="C120" s="3"/>
-      <c r="D120" s="3"/>
-      <c r="E120" s="3"/>
-      <c r="F120" s="3"/>
+      <c r="A120" s="4"/>
+      <c r="B120" s="4"/>
+      <c r="C120" s="4"/>
+      <c r="D120" s="4"/>
+      <c r="E120" s="4"/>
+      <c r="F120" s="4"/>
       <c r="G120" s="1"/>
       <c r="H120" s="1"/>
     </row>
     <row r="121" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="4"/>
-      <c r="B121" s="4"/>
-      <c r="C121" s="4"/>
-      <c r="D121" s="4"/>
-      <c r="E121" s="4"/>
-      <c r="F121" s="4"/>
+      <c r="A121" s="5"/>
+      <c r="B121" s="5"/>
+      <c r="C121" s="5"/>
+      <c r="D121" s="5"/>
+      <c r="E121" s="5"/>
+      <c r="F121" s="5"/>
       <c r="G121" s="1"/>
       <c r="H121" s="1"/>
     </row>
     <row r="122" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="8" t="s">
+      <c r="A122" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B122" s="7"/>
-      <c r="C122" s="2" t="s">
+      <c r="B122" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C122" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="D122" s="6" t="s">
+      <c r="D122" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E122" s="5" t="s">
+      <c r="E122" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F122" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G122" s="9" t="s">
+      <c r="F122" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G122" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="H122" s="9" t="s">
+      <c r="H122" s="2" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="3"/>
-      <c r="B123" s="3"/>
-      <c r="C123" s="3"/>
-      <c r="D123" s="3"/>
-      <c r="E123" s="3"/>
-      <c r="F123" s="3"/>
+      <c r="A123" s="4"/>
+      <c r="B123" s="4"/>
+      <c r="C123" s="4"/>
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+      <c r="F123" s="4"/>
       <c r="G123" s="1"/>
       <c r="H123" s="1"/>
     </row>
     <row r="124" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="3"/>
-      <c r="B124" s="3"/>
-      <c r="C124" s="3"/>
-      <c r="D124" s="3"/>
-      <c r="E124" s="3"/>
-      <c r="F124" s="3"/>
+      <c r="A124" s="4"/>
+      <c r="B124" s="4"/>
+      <c r="C124" s="4"/>
+      <c r="D124" s="4"/>
+      <c r="E124" s="4"/>
+      <c r="F124" s="4"/>
       <c r="G124" s="1"/>
       <c r="H124" s="1"/>
     </row>
     <row r="125" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="4"/>
-      <c r="B125" s="4"/>
-      <c r="C125" s="4"/>
-      <c r="D125" s="4"/>
-      <c r="E125" s="4"/>
-      <c r="F125" s="4"/>
+      <c r="A125" s="5"/>
+      <c r="B125" s="5"/>
+      <c r="C125" s="5"/>
+      <c r="D125" s="5"/>
+      <c r="E125" s="5"/>
+      <c r="F125" s="5"/>
       <c r="G125" s="1"/>
       <c r="H125" s="1"/>
     </row>
     <row r="126" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="8" t="s">
+      <c r="A126" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B126" s="7"/>
-      <c r="C126" s="2" t="s">
+      <c r="B126" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C126" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="D126" s="6" t="s">
+      <c r="D126" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E126" s="5" t="s">
+      <c r="E126" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="F126" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G126" s="9" t="s">
+      <c r="F126" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G126" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="H126" s="9" t="s">
+      <c r="H126" s="2" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="3"/>
-      <c r="B127" s="3"/>
-      <c r="C127" s="3"/>
-      <c r="D127" s="3"/>
-      <c r="E127" s="3"/>
-      <c r="F127" s="3"/>
+      <c r="A127" s="4"/>
+      <c r="B127" s="4"/>
+      <c r="C127" s="4"/>
+      <c r="D127" s="4"/>
+      <c r="E127" s="4"/>
+      <c r="F127" s="4"/>
       <c r="G127" s="1"/>
-      <c r="H127" s="9"/>
+      <c r="H127" s="2"/>
     </row>
     <row r="128" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="3"/>
-      <c r="B128" s="3"/>
-      <c r="C128" s="3"/>
-      <c r="D128" s="3"/>
-      <c r="E128" s="3"/>
-      <c r="F128" s="3"/>
+      <c r="A128" s="4"/>
+      <c r="B128" s="4"/>
+      <c r="C128" s="4"/>
+      <c r="D128" s="4"/>
+      <c r="E128" s="4"/>
+      <c r="F128" s="4"/>
       <c r="G128" s="1"/>
       <c r="H128" s="1"/>
     </row>
     <row r="129" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="4"/>
-      <c r="B129" s="4"/>
-      <c r="C129" s="4"/>
-      <c r="D129" s="4"/>
-      <c r="E129" s="4"/>
-      <c r="F129" s="4"/>
+      <c r="A129" s="5"/>
+      <c r="B129" s="5"/>
+      <c r="C129" s="5"/>
+      <c r="D129" s="5"/>
+      <c r="E129" s="5"/>
+      <c r="F129" s="5"/>
       <c r="G129" s="1"/>
       <c r="H129" s="1"/>
     </row>
     <row r="130" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="8" t="s">
+      <c r="A130" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B130" s="7"/>
-      <c r="C130" s="2" t="s">
+      <c r="B130" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C130" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="D130" s="6" t="s">
+      <c r="D130" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E130" s="5" t="s">
+      <c r="E130" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="F130" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G130" s="9" t="s">
+      <c r="F130" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G130" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="H130" s="9" t="s">
+      <c r="H130" s="2" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="3"/>
-      <c r="B131" s="3"/>
-      <c r="C131" s="3"/>
-      <c r="D131" s="3"/>
-      <c r="E131" s="3"/>
-      <c r="F131" s="3"/>
+      <c r="A131" s="4"/>
+      <c r="B131" s="4"/>
+      <c r="C131" s="4"/>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
       <c r="G131" s="1"/>
       <c r="H131" s="1"/>
     </row>
     <row r="132" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A132" s="3"/>
-      <c r="B132" s="3"/>
-      <c r="C132" s="3"/>
-      <c r="D132" s="3"/>
-      <c r="E132" s="3"/>
-      <c r="F132" s="3"/>
+      <c r="A132" s="4"/>
+      <c r="B132" s="4"/>
+      <c r="C132" s="4"/>
+      <c r="D132" s="4"/>
+      <c r="E132" s="4"/>
+      <c r="F132" s="4"/>
       <c r="G132" s="1"/>
       <c r="H132" s="1"/>
     </row>
     <row r="133" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A133" s="4"/>
-      <c r="B133" s="4"/>
-      <c r="C133" s="4"/>
-      <c r="D133" s="4"/>
-      <c r="E133" s="4"/>
-      <c r="F133" s="4"/>
+      <c r="A133" s="5"/>
+      <c r="B133" s="5"/>
+      <c r="C133" s="5"/>
+      <c r="D133" s="5"/>
+      <c r="E133" s="5"/>
+      <c r="F133" s="5"/>
       <c r="G133" s="1"/>
       <c r="H133" s="1"/>
     </row>
     <row r="134" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="8" t="s">
+      <c r="A134" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B134" s="7"/>
-      <c r="C134" s="2" t="s">
+      <c r="B134" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C134" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="D134" s="6" t="s">
+      <c r="D134" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="E134" s="5" t="s">
+      <c r="E134" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="F134" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G134" s="9" t="s">
+      <c r="F134" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G134" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H134" s="9" t="s">
+      <c r="H134" s="2" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="3"/>
-      <c r="B135" s="3"/>
-      <c r="C135" s="3"/>
-      <c r="D135" s="3"/>
-      <c r="E135" s="3"/>
-      <c r="F135" s="3"/>
-      <c r="G135" s="9" t="s">
+      <c r="A135" s="4"/>
+      <c r="B135" s="4"/>
+      <c r="C135" s="4"/>
+      <c r="D135" s="4"/>
+      <c r="E135" s="4"/>
+      <c r="F135" s="4"/>
+      <c r="G135" s="2" t="s">
         <v>236</v>
       </c>
       <c r="H135" s="1"/>
     </row>
     <row r="136" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="3"/>
-      <c r="B136" s="3"/>
-      <c r="C136" s="3"/>
-      <c r="D136" s="3"/>
-      <c r="E136" s="3"/>
-      <c r="F136" s="3"/>
-      <c r="G136" s="9" t="s">
+      <c r="A136" s="4"/>
+      <c r="B136" s="4"/>
+      <c r="C136" s="4"/>
+      <c r="D136" s="4"/>
+      <c r="E136" s="4"/>
+      <c r="F136" s="4"/>
+      <c r="G136" s="2" t="s">
         <v>265</v>
       </c>
       <c r="H136" s="1"/>
     </row>
     <row r="137" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="4"/>
-      <c r="B137" s="4"/>
-      <c r="C137" s="4"/>
-      <c r="D137" s="4"/>
-      <c r="E137" s="4"/>
-      <c r="F137" s="4"/>
+      <c r="A137" s="5"/>
+      <c r="B137" s="5"/>
+      <c r="C137" s="5"/>
+      <c r="D137" s="5"/>
+      <c r="E137" s="5"/>
+      <c r="F137" s="5"/>
       <c r="G137" s="1"/>
       <c r="H137" s="1"/>
     </row>
     <row r="138" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="8" t="s">
+      <c r="A138" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B138" s="7"/>
-      <c r="C138" s="2" t="s">
+      <c r="B138" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C138" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="D138" s="6" t="s">
+      <c r="D138" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="E138" s="5" t="s">
+      <c r="E138" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="F138" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G138" s="9" t="s">
+      <c r="F138" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G138" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="H138" s="9" t="s">
+      <c r="H138" s="2" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="139" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A139" s="3"/>
-      <c r="B139" s="3"/>
-      <c r="C139" s="3"/>
-      <c r="D139" s="3"/>
-      <c r="E139" s="3"/>
-      <c r="F139" s="3"/>
-      <c r="G139" s="9" t="s">
+      <c r="A139" s="4"/>
+      <c r="B139" s="4"/>
+      <c r="C139" s="4"/>
+      <c r="D139" s="4"/>
+      <c r="E139" s="4"/>
+      <c r="F139" s="4"/>
+      <c r="G139" s="2" t="s">
         <v>236</v>
       </c>
       <c r="H139" s="1"/>
     </row>
     <row r="140" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="3"/>
-      <c r="B140" s="3"/>
-      <c r="C140" s="3"/>
-      <c r="D140" s="3"/>
-      <c r="E140" s="3"/>
-      <c r="F140" s="3"/>
-      <c r="G140" s="9"/>
+      <c r="A140" s="4"/>
+      <c r="B140" s="4"/>
+      <c r="C140" s="4"/>
+      <c r="D140" s="4"/>
+      <c r="E140" s="4"/>
+      <c r="F140" s="4"/>
+      <c r="G140" s="2"/>
       <c r="H140" s="1"/>
     </row>
     <row r="141" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A141" s="4"/>
-      <c r="B141" s="4"/>
-      <c r="C141" s="4"/>
-      <c r="D141" s="4"/>
-      <c r="E141" s="4"/>
-      <c r="F141" s="4"/>
+      <c r="A141" s="5"/>
+      <c r="B141" s="5"/>
+      <c r="C141" s="5"/>
+      <c r="D141" s="5"/>
+      <c r="E141" s="5"/>
+      <c r="F141" s="5"/>
       <c r="G141" s="1"/>
       <c r="H141" s="1"/>
     </row>
     <row r="142" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="8" t="s">
+      <c r="A142" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B142" s="7"/>
-      <c r="C142" s="2" t="s">
+      <c r="B142" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C142" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="D142" s="6" t="s">
+      <c r="D142" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="E142" s="5" t="s">
+      <c r="E142" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F142" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G142" s="9" t="s">
+      <c r="F142" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G142" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="H142" s="9" t="s">
+      <c r="H142" s="2" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A143" s="3"/>
-      <c r="B143" s="3"/>
-      <c r="C143" s="3"/>
-      <c r="D143" s="3"/>
-      <c r="E143" s="3"/>
-      <c r="F143" s="3"/>
-      <c r="G143" s="9" t="s">
+      <c r="A143" s="4"/>
+      <c r="B143" s="4"/>
+      <c r="C143" s="4"/>
+      <c r="D143" s="4"/>
+      <c r="E143" s="4"/>
+      <c r="F143" s="4"/>
+      <c r="G143" s="2" t="s">
         <v>256</v>
       </c>
       <c r="H143" s="1"/>
     </row>
     <row r="144" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="3"/>
-      <c r="B144" s="3"/>
-      <c r="C144" s="3"/>
-      <c r="D144" s="3"/>
-      <c r="E144" s="3"/>
-      <c r="F144" s="3"/>
+      <c r="A144" s="4"/>
+      <c r="B144" s="4"/>
+      <c r="C144" s="4"/>
+      <c r="D144" s="4"/>
+      <c r="E144" s="4"/>
+      <c r="F144" s="4"/>
       <c r="G144" s="1"/>
       <c r="H144" s="1"/>
     </row>
     <row r="145" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="4"/>
-      <c r="B145" s="4"/>
-      <c r="C145" s="4"/>
-      <c r="D145" s="4"/>
-      <c r="E145" s="4"/>
-      <c r="F145" s="4"/>
+      <c r="A145" s="5"/>
+      <c r="B145" s="5"/>
+      <c r="C145" s="5"/>
+      <c r="D145" s="5"/>
+      <c r="E145" s="5"/>
+      <c r="F145" s="5"/>
       <c r="G145" s="1"/>
       <c r="H145" s="1"/>
     </row>
     <row r="146" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="8" t="s">
+      <c r="A146" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B146" s="7"/>
-      <c r="C146" s="2" t="s">
+      <c r="B146" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C146" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="D146" s="6" t="s">
+      <c r="D146" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="E146" s="5" t="s">
+      <c r="E146" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="F146" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G146" s="9" t="s">
+      <c r="F146" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G146" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="H146" s="9" t="s">
+      <c r="H146" s="2" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="147" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="3"/>
-      <c r="B147" s="3"/>
-      <c r="C147" s="3"/>
-      <c r="D147" s="3"/>
-      <c r="E147" s="3"/>
-      <c r="F147" s="3"/>
-      <c r="G147" s="9" t="s">
+      <c r="A147" s="4"/>
+      <c r="B147" s="4"/>
+      <c r="C147" s="4"/>
+      <c r="D147" s="4"/>
+      <c r="E147" s="4"/>
+      <c r="F147" s="4"/>
+      <c r="G147" s="2" t="s">
         <v>270</v>
       </c>
       <c r="H147" s="1"/>
     </row>
     <row r="148" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="3"/>
-      <c r="B148" s="3"/>
-      <c r="C148" s="3"/>
-      <c r="D148" s="3"/>
-      <c r="E148" s="3"/>
-      <c r="F148" s="3"/>
+      <c r="A148" s="4"/>
+      <c r="B148" s="4"/>
+      <c r="C148" s="4"/>
+      <c r="D148" s="4"/>
+      <c r="E148" s="4"/>
+      <c r="F148" s="4"/>
       <c r="G148" s="1"/>
       <c r="H148" s="1"/>
     </row>
     <row r="149" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="4"/>
-      <c r="B149" s="4"/>
-      <c r="C149" s="4"/>
-      <c r="D149" s="4"/>
-      <c r="E149" s="4"/>
-      <c r="F149" s="4"/>
+      <c r="A149" s="5"/>
+      <c r="B149" s="5"/>
+      <c r="C149" s="5"/>
+      <c r="D149" s="5"/>
+      <c r="E149" s="5"/>
+      <c r="F149" s="5"/>
       <c r="G149" s="1"/>
       <c r="H149" s="1"/>
     </row>
     <row r="150" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="8" t="s">
+      <c r="A150" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B150" s="7"/>
-      <c r="C150" s="2" t="s">
+      <c r="B150" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C150" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="D150" s="6" t="s">
+      <c r="D150" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="E150" s="5" t="s">
+      <c r="E150" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F150" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G150" s="9" t="s">
+      <c r="F150" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G150" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H150" s="9" t="s">
+      <c r="H150" s="2" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A151" s="3"/>
-      <c r="B151" s="3"/>
-      <c r="C151" s="3"/>
-      <c r="D151" s="3"/>
-      <c r="E151" s="3"/>
-      <c r="F151" s="3"/>
-      <c r="G151" s="9" t="s">
+      <c r="A151" s="4"/>
+      <c r="B151" s="4"/>
+      <c r="C151" s="4"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="4"/>
+      <c r="F151" s="4"/>
+      <c r="G151" s="2" t="s">
         <v>214</v>
       </c>
       <c r="H151" s="1"/>
     </row>
     <row r="152" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A152" s="3"/>
-      <c r="B152" s="3"/>
-      <c r="C152" s="3"/>
-      <c r="D152" s="3"/>
-      <c r="E152" s="3"/>
-      <c r="F152" s="3"/>
-      <c r="G152" s="9" t="s">
+      <c r="A152" s="4"/>
+      <c r="B152" s="4"/>
+      <c r="C152" s="4"/>
+      <c r="D152" s="4"/>
+      <c r="E152" s="4"/>
+      <c r="F152" s="4"/>
+      <c r="G152" s="2" t="s">
         <v>270</v>
       </c>
       <c r="H152" s="1"/>
     </row>
     <row r="153" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="4"/>
-      <c r="B153" s="4"/>
-      <c r="C153" s="4"/>
-      <c r="D153" s="4"/>
-      <c r="E153" s="4"/>
-      <c r="F153" s="4"/>
+      <c r="A153" s="5"/>
+      <c r="B153" s="5"/>
+      <c r="C153" s="5"/>
+      <c r="D153" s="5"/>
+      <c r="E153" s="5"/>
+      <c r="F153" s="5"/>
       <c r="G153" s="1"/>
       <c r="H153" s="1"/>
     </row>
     <row r="154" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="8" t="s">
+      <c r="A154" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="B154" s="7"/>
-      <c r="C154" s="2" t="s">
+      <c r="B154" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C154" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="D154" s="6" t="s">
+      <c r="D154" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="E154" s="5" t="s">
+      <c r="E154" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="F154" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G154" s="9" t="s">
+      <c r="F154" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G154" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="H154" s="9" t="s">
+      <c r="H154" s="2" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="3"/>
-      <c r="B155" s="3"/>
-      <c r="C155" s="3"/>
-      <c r="D155" s="3"/>
-      <c r="E155" s="3"/>
-      <c r="F155" s="3"/>
-      <c r="G155" s="9" t="s">
+      <c r="A155" s="4"/>
+      <c r="B155" s="4"/>
+      <c r="C155" s="4"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="4"/>
+      <c r="F155" s="4"/>
+      <c r="G155" s="2" t="s">
         <v>240</v>
       </c>
       <c r="H155" s="1"/>
     </row>
     <row r="156" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A156" s="3"/>
-      <c r="B156" s="3"/>
-      <c r="C156" s="3"/>
-      <c r="D156" s="3"/>
-      <c r="E156" s="3"/>
-      <c r="F156" s="3"/>
+      <c r="A156" s="4"/>
+      <c r="B156" s="4"/>
+      <c r="C156" s="4"/>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4"/>
+      <c r="F156" s="4"/>
       <c r="G156" s="1"/>
       <c r="H156" s="1"/>
     </row>
     <row r="157" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A157" s="4"/>
-      <c r="B157" s="4"/>
-      <c r="C157" s="4"/>
-      <c r="D157" s="4"/>
-      <c r="E157" s="4"/>
-      <c r="F157" s="4"/>
+      <c r="A157" s="5"/>
+      <c r="B157" s="5"/>
+      <c r="C157" s="5"/>
+      <c r="D157" s="5"/>
+      <c r="E157" s="5"/>
+      <c r="F157" s="5"/>
       <c r="G157" s="1"/>
       <c r="H157" s="1"/>
     </row>
     <row r="158" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A158" s="8" t="s">
+      <c r="A158" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B158" s="7"/>
-      <c r="C158" s="2" t="s">
+      <c r="B158" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C158" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="D158" s="6" t="s">
+      <c r="D158" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="E158" s="5" t="s">
+      <c r="E158" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="F158" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G158" s="9" t="s">
+      <c r="F158" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G158" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="H158" s="9" t="s">
+      <c r="H158" s="2" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A159" s="3"/>
-      <c r="B159" s="3"/>
-      <c r="C159" s="3"/>
-      <c r="D159" s="3"/>
-      <c r="E159" s="3"/>
-      <c r="F159" s="3"/>
-      <c r="G159" s="9" t="s">
+      <c r="A159" s="4"/>
+      <c r="B159" s="4"/>
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="4"/>
+      <c r="F159" s="4"/>
+      <c r="G159" s="2" t="s">
         <v>233</v>
       </c>
       <c r="H159" s="1"/>
     </row>
     <row r="160" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="3"/>
-      <c r="B160" s="3"/>
-      <c r="C160" s="3"/>
-      <c r="D160" s="3"/>
-      <c r="E160" s="3"/>
-      <c r="F160" s="3"/>
+      <c r="A160" s="4"/>
+      <c r="B160" s="4"/>
+      <c r="C160" s="4"/>
+      <c r="D160" s="4"/>
+      <c r="E160" s="4"/>
+      <c r="F160" s="4"/>
       <c r="G160" s="1"/>
       <c r="H160" s="1"/>
     </row>
     <row r="161" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A161" s="4"/>
-      <c r="B161" s="4"/>
-      <c r="C161" s="4"/>
-      <c r="D161" s="4"/>
-      <c r="E161" s="4"/>
-      <c r="F161" s="4"/>
+      <c r="A161" s="5"/>
+      <c r="B161" s="5"/>
+      <c r="C161" s="5"/>
+      <c r="D161" s="5"/>
+      <c r="E161" s="5"/>
+      <c r="F161" s="5"/>
       <c r="G161" s="1"/>
       <c r="H161" s="1"/>
     </row>
     <row r="162" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="8" t="s">
+      <c r="A162" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B162" s="7"/>
-      <c r="C162" s="2" t="s">
+      <c r="B162" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C162" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="D162" s="6" t="s">
+      <c r="D162" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="E162" s="5" t="s">
+      <c r="E162" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="F162" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G162" s="9" t="s">
+      <c r="F162" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G162" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="H162" s="9" t="s">
+      <c r="H162" s="2" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A163" s="3"/>
-      <c r="B163" s="3"/>
-      <c r="C163" s="3"/>
-      <c r="D163" s="3"/>
-      <c r="E163" s="3"/>
-      <c r="F163" s="3"/>
-      <c r="G163" s="9" t="s">
+      <c r="A163" s="4"/>
+      <c r="B163" s="4"/>
+      <c r="C163" s="4"/>
+      <c r="D163" s="4"/>
+      <c r="E163" s="4"/>
+      <c r="F163" s="4"/>
+      <c r="G163" s="2" t="s">
         <v>256</v>
       </c>
       <c r="H163" s="1"/>
     </row>
     <row r="164" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A164" s="3"/>
-      <c r="B164" s="3"/>
-      <c r="C164" s="3"/>
-      <c r="D164" s="3"/>
-      <c r="E164" s="3"/>
-      <c r="F164" s="3"/>
+      <c r="A164" s="4"/>
+      <c r="B164" s="4"/>
+      <c r="C164" s="4"/>
+      <c r="D164" s="4"/>
+      <c r="E164" s="4"/>
+      <c r="F164" s="4"/>
       <c r="G164" s="1"/>
       <c r="H164" s="1"/>
     </row>
     <row r="165" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A165" s="4"/>
-      <c r="B165" s="4"/>
-      <c r="C165" s="4"/>
-      <c r="D165" s="4"/>
-      <c r="E165" s="4"/>
-      <c r="F165" s="4"/>
+      <c r="A165" s="5"/>
+      <c r="B165" s="5"/>
+      <c r="C165" s="5"/>
+      <c r="D165" s="5"/>
+      <c r="E165" s="5"/>
+      <c r="F165" s="5"/>
       <c r="G165" s="1"/>
       <c r="H165" s="1"/>
     </row>
     <row r="166" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A166" s="8" t="s">
+      <c r="A166" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B166" s="7"/>
-      <c r="C166" s="2" t="s">
+      <c r="B166" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C166" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="D166" s="6" t="s">
+      <c r="D166" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="E166" s="5" t="s">
+      <c r="E166" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="F166" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G166" s="9" t="s">
+      <c r="F166" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G166" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="H166" s="9" t="s">
+      <c r="H166" s="2" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="167" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A167" s="3"/>
-      <c r="B167" s="3"/>
-      <c r="C167" s="3"/>
-      <c r="D167" s="3"/>
-      <c r="E167" s="3"/>
-      <c r="F167" s="3"/>
-      <c r="G167" s="9" t="s">
+      <c r="A167" s="4"/>
+      <c r="B167" s="4"/>
+      <c r="C167" s="4"/>
+      <c r="D167" s="4"/>
+      <c r="E167" s="4"/>
+      <c r="F167" s="4"/>
+      <c r="G167" s="2" t="s">
         <v>256</v>
       </c>
       <c r="H167" s="1"/>
     </row>
     <row r="168" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A168" s="3"/>
-      <c r="B168" s="3"/>
-      <c r="C168" s="3"/>
-      <c r="D168" s="3"/>
-      <c r="E168" s="3"/>
-      <c r="F168" s="3"/>
+      <c r="A168" s="4"/>
+      <c r="B168" s="4"/>
+      <c r="C168" s="4"/>
+      <c r="D168" s="4"/>
+      <c r="E168" s="4"/>
+      <c r="F168" s="4"/>
       <c r="G168" s="1"/>
       <c r="H168" s="1"/>
     </row>
     <row r="169" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A169" s="4"/>
-      <c r="B169" s="4"/>
-      <c r="C169" s="4"/>
-      <c r="D169" s="4"/>
-      <c r="E169" s="4"/>
-      <c r="F169" s="4"/>
+      <c r="A169" s="5"/>
+      <c r="B169" s="5"/>
+      <c r="C169" s="5"/>
+      <c r="D169" s="5"/>
+      <c r="E169" s="5"/>
+      <c r="F169" s="5"/>
       <c r="G169" s="1"/>
       <c r="H169" s="1"/>
     </row>
     <row r="170" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="8" t="s">
+      <c r="A170" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B170" s="7"/>
-      <c r="C170" s="2" t="s">
+      <c r="B170" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C170" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="D170" s="6" t="s">
+      <c r="D170" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="E170" s="5" t="s">
+      <c r="E170" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="F170" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G170" s="9" t="s">
+      <c r="F170" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G170" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="H170" s="9" t="s">
+      <c r="H170" s="2" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="171" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A171" s="3"/>
-      <c r="B171" s="3"/>
-      <c r="C171" s="3"/>
-      <c r="D171" s="3"/>
-      <c r="E171" s="3"/>
-      <c r="F171" s="3"/>
+      <c r="A171" s="4"/>
+      <c r="B171" s="4"/>
+      <c r="C171" s="4"/>
+      <c r="D171" s="4"/>
+      <c r="E171" s="4"/>
+      <c r="F171" s="4"/>
       <c r="G171" s="1"/>
       <c r="H171" s="1"/>
     </row>
     <row r="172" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A172" s="3"/>
-      <c r="B172" s="3"/>
-      <c r="C172" s="3"/>
-      <c r="D172" s="3"/>
-      <c r="E172" s="3"/>
-      <c r="F172" s="3"/>
+      <c r="A172" s="4"/>
+      <c r="B172" s="4"/>
+      <c r="C172" s="4"/>
+      <c r="D172" s="4"/>
+      <c r="E172" s="4"/>
+      <c r="F172" s="4"/>
       <c r="G172" s="1"/>
       <c r="H172" s="1"/>
     </row>
     <row r="173" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A173" s="4"/>
-      <c r="B173" s="4"/>
-      <c r="C173" s="4"/>
-      <c r="D173" s="4"/>
-      <c r="E173" s="4"/>
-      <c r="F173" s="4"/>
+      <c r="A173" s="5"/>
+      <c r="B173" s="5"/>
+      <c r="C173" s="5"/>
+      <c r="D173" s="5"/>
+      <c r="E173" s="5"/>
+      <c r="F173" s="5"/>
       <c r="G173" s="1"/>
       <c r="H173" s="1"/>
     </row>
     <row r="174" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A174" s="8" t="s">
+      <c r="A174" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B174" s="7"/>
-      <c r="C174" s="2" t="s">
+      <c r="B174" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C174" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="D174" s="6" t="s">
+      <c r="D174" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="E174" s="5" t="s">
+      <c r="E174" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="F174" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G174" s="9" t="s">
+      <c r="F174" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G174" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="H174" s="9" t="s">
+      <c r="H174" s="2" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A175" s="3"/>
-      <c r="B175" s="3"/>
-      <c r="C175" s="3"/>
-      <c r="D175" s="3"/>
-      <c r="E175" s="3"/>
-      <c r="F175" s="3"/>
-      <c r="G175" s="9" t="s">
+      <c r="A175" s="4"/>
+      <c r="B175" s="4"/>
+      <c r="C175" s="4"/>
+      <c r="D175" s="4"/>
+      <c r="E175" s="4"/>
+      <c r="F175" s="4"/>
+      <c r="G175" s="2" t="s">
         <v>233</v>
       </c>
       <c r="H175" s="1"/>
     </row>
     <row r="176" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A176" s="3"/>
-      <c r="B176" s="3"/>
-      <c r="C176" s="3"/>
-      <c r="D176" s="3"/>
-      <c r="E176" s="3"/>
-      <c r="F176" s="3"/>
+      <c r="A176" s="4"/>
+      <c r="B176" s="4"/>
+      <c r="C176" s="4"/>
+      <c r="D176" s="4"/>
+      <c r="E176" s="4"/>
+      <c r="F176" s="4"/>
       <c r="G176" s="1"/>
       <c r="H176" s="1"/>
     </row>
     <row r="177" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A177" s="4"/>
-      <c r="B177" s="4"/>
-      <c r="C177" s="4"/>
-      <c r="D177" s="4"/>
-      <c r="E177" s="4"/>
-      <c r="F177" s="4"/>
+      <c r="A177" s="5"/>
+      <c r="B177" s="5"/>
+      <c r="C177" s="5"/>
+      <c r="D177" s="5"/>
+      <c r="E177" s="5"/>
+      <c r="F177" s="5"/>
       <c r="G177" s="1"/>
       <c r="H177" s="1"/>
     </row>
     <row r="178" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A178" s="8" t="s">
+      <c r="A178" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B178" s="7"/>
-      <c r="C178" s="2" t="s">
+      <c r="B178" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C178" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="D178" s="6" t="s">
+      <c r="D178" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="E178" s="5" t="s">
+      <c r="E178" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="F178" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G178" s="9" t="s">
+      <c r="F178" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G178" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="H178" s="9" t="s">
+      <c r="H178" s="2" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="179" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A179" s="3"/>
-      <c r="B179" s="3"/>
-      <c r="C179" s="3"/>
-      <c r="D179" s="3"/>
-      <c r="E179" s="3"/>
-      <c r="F179" s="3"/>
+      <c r="A179" s="4"/>
+      <c r="B179" s="4"/>
+      <c r="C179" s="4"/>
+      <c r="D179" s="4"/>
+      <c r="E179" s="4"/>
+      <c r="F179" s="4"/>
       <c r="G179" s="1"/>
       <c r="H179" s="1"/>
     </row>
     <row r="180" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A180" s="3"/>
-      <c r="B180" s="3"/>
-      <c r="C180" s="3"/>
-      <c r="D180" s="3"/>
-      <c r="E180" s="3"/>
-      <c r="F180" s="3"/>
+      <c r="A180" s="4"/>
+      <c r="B180" s="4"/>
+      <c r="C180" s="4"/>
+      <c r="D180" s="4"/>
+      <c r="E180" s="4"/>
+      <c r="F180" s="4"/>
       <c r="G180" s="1"/>
       <c r="H180" s="1"/>
     </row>
     <row r="181" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A181" s="4"/>
-      <c r="B181" s="4"/>
-      <c r="C181" s="4"/>
-      <c r="D181" s="4"/>
-      <c r="E181" s="4"/>
-      <c r="F181" s="4"/>
+      <c r="A181" s="5"/>
+      <c r="B181" s="5"/>
+      <c r="C181" s="5"/>
+      <c r="D181" s="5"/>
+      <c r="E181" s="5"/>
+      <c r="F181" s="5"/>
       <c r="G181" s="1"/>
       <c r="H181" s="1"/>
     </row>
     <row r="182" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A182" s="8" t="s">
+      <c r="A182" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B182" s="7"/>
-      <c r="C182" s="2" t="s">
+      <c r="B182" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C182" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="D182" s="6" t="s">
+      <c r="D182" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E182" s="5" t="s">
+      <c r="E182" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="F182" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G182" s="9" t="s">
+      <c r="F182" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G182" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="H182" s="9" t="s">
+      <c r="H182" s="2" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="183" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A183" s="3"/>
-      <c r="B183" s="3"/>
-      <c r="C183" s="3"/>
-      <c r="D183" s="3"/>
-      <c r="E183" s="3"/>
-      <c r="F183" s="3"/>
+      <c r="A183" s="4"/>
+      <c r="B183" s="4"/>
+      <c r="C183" s="4"/>
+      <c r="D183" s="4"/>
+      <c r="E183" s="4"/>
+      <c r="F183" s="4"/>
       <c r="G183" s="1"/>
       <c r="H183" s="1"/>
     </row>
     <row r="184" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A184" s="3"/>
-      <c r="B184" s="3"/>
-      <c r="C184" s="3"/>
-      <c r="D184" s="3"/>
-      <c r="E184" s="3"/>
-      <c r="F184" s="3"/>
+      <c r="A184" s="4"/>
+      <c r="B184" s="4"/>
+      <c r="C184" s="4"/>
+      <c r="D184" s="4"/>
+      <c r="E184" s="4"/>
+      <c r="F184" s="4"/>
       <c r="G184" s="1"/>
       <c r="H184" s="1"/>
     </row>
     <row r="185" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A185" s="4"/>
-      <c r="B185" s="4"/>
-      <c r="C185" s="4"/>
-      <c r="D185" s="4"/>
-      <c r="E185" s="4"/>
-      <c r="F185" s="4"/>
+      <c r="A185" s="5"/>
+      <c r="B185" s="5"/>
+      <c r="C185" s="5"/>
+      <c r="D185" s="5"/>
+      <c r="E185" s="5"/>
+      <c r="F185" s="5"/>
       <c r="G185" s="1"/>
       <c r="H185" s="1"/>
     </row>
     <row r="186" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A186" s="8" t="s">
+      <c r="A186" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B186" s="7"/>
-      <c r="C186" s="2" t="s">
+      <c r="B186" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C186" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="D186" s="6" t="s">
+      <c r="D186" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="E186" s="5" t="s">
+      <c r="E186" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="F186" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G186" s="9" t="s">
+      <c r="F186" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G186" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="H186" s="9" t="s">
+      <c r="H186" s="2" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="187" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A187" s="3"/>
-      <c r="B187" s="3"/>
-      <c r="C187" s="3"/>
-      <c r="D187" s="3"/>
-      <c r="E187" s="3"/>
-      <c r="F187" s="3"/>
-      <c r="G187" s="9" t="s">
+      <c r="A187" s="4"/>
+      <c r="B187" s="4"/>
+      <c r="C187" s="4"/>
+      <c r="D187" s="4"/>
+      <c r="E187" s="4"/>
+      <c r="F187" s="4"/>
+      <c r="G187" s="2" t="s">
         <v>270</v>
       </c>
       <c r="H187" s="1"/>
     </row>
     <row r="188" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A188" s="3"/>
-      <c r="B188" s="3"/>
-      <c r="C188" s="3"/>
-      <c r="D188" s="3"/>
-      <c r="E188" s="3"/>
-      <c r="F188" s="3"/>
+      <c r="A188" s="4"/>
+      <c r="B188" s="4"/>
+      <c r="C188" s="4"/>
+      <c r="D188" s="4"/>
+      <c r="E188" s="4"/>
+      <c r="F188" s="4"/>
       <c r="G188" s="1"/>
       <c r="H188" s="1"/>
     </row>
     <row r="189" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A189" s="4"/>
-      <c r="B189" s="4"/>
-      <c r="C189" s="4"/>
-      <c r="D189" s="4"/>
-      <c r="E189" s="4"/>
-      <c r="F189" s="4"/>
+      <c r="A189" s="5"/>
+      <c r="B189" s="5"/>
+      <c r="C189" s="5"/>
+      <c r="D189" s="5"/>
+      <c r="E189" s="5"/>
+      <c r="F189" s="5"/>
       <c r="G189" s="1"/>
       <c r="H189" s="1"/>
     </row>
     <row r="190" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="8" t="s">
+      <c r="A190" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B190" s="7"/>
-      <c r="C190" s="2" t="s">
+      <c r="B190" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C190" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="D190" s="6" t="s">
+      <c r="D190" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="E190" s="5" t="s">
+      <c r="E190" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="F190" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G190" s="9" t="s">
+      <c r="F190" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G190" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H190" s="9" t="s">
+      <c r="H190" s="2" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="191" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A191" s="3"/>
-      <c r="B191" s="3"/>
-      <c r="C191" s="3"/>
-      <c r="D191" s="3"/>
-      <c r="E191" s="3"/>
-      <c r="F191" s="3"/>
-      <c r="G191" s="9" t="s">
+      <c r="A191" s="4"/>
+      <c r="B191" s="4"/>
+      <c r="C191" s="4"/>
+      <c r="D191" s="4"/>
+      <c r="E191" s="4"/>
+      <c r="F191" s="4"/>
+      <c r="G191" s="2" t="s">
         <v>282</v>
       </c>
       <c r="H191" s="1"/>
     </row>
     <row r="192" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A192" s="3"/>
-      <c r="B192" s="3"/>
-      <c r="C192" s="3"/>
-      <c r="D192" s="3"/>
-      <c r="E192" s="3"/>
-      <c r="F192" s="3"/>
+      <c r="A192" s="4"/>
+      <c r="B192" s="4"/>
+      <c r="C192" s="4"/>
+      <c r="D192" s="4"/>
+      <c r="E192" s="4"/>
+      <c r="F192" s="4"/>
       <c r="G192" s="1"/>
       <c r="H192" s="1"/>
     </row>
     <row r="193" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A193" s="4"/>
-      <c r="B193" s="4"/>
-      <c r="C193" s="4"/>
-      <c r="D193" s="4"/>
-      <c r="E193" s="4"/>
-      <c r="F193" s="4"/>
+      <c r="A193" s="5"/>
+      <c r="B193" s="5"/>
+      <c r="C193" s="5"/>
+      <c r="D193" s="5"/>
+      <c r="E193" s="5"/>
+      <c r="F193" s="5"/>
       <c r="G193" s="1"/>
       <c r="H193" s="1"/>
     </row>
     <row r="194" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A194" s="8" t="s">
+      <c r="A194" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B194" s="7"/>
-      <c r="C194" s="2" t="s">
+      <c r="B194" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C194" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="D194" s="6" t="s">
+      <c r="D194" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="E194" s="5" t="s">
+      <c r="E194" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="F194" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G194" s="9" t="s">
+      <c r="F194" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G194" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="H194" s="9" t="s">
+      <c r="H194" s="2" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="195" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A195" s="3"/>
-      <c r="B195" s="3"/>
-      <c r="C195" s="3"/>
-      <c r="D195" s="3"/>
-      <c r="E195" s="3"/>
-      <c r="F195" s="3"/>
-      <c r="G195" s="9" t="s">
+      <c r="A195" s="4"/>
+      <c r="B195" s="4"/>
+      <c r="C195" s="4"/>
+      <c r="D195" s="4"/>
+      <c r="E195" s="4"/>
+      <c r="F195" s="4"/>
+      <c r="G195" s="2" t="s">
         <v>285</v>
       </c>
       <c r="H195" s="1"/>
     </row>
     <row r="196" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A196" s="3"/>
-      <c r="B196" s="3"/>
-      <c r="C196" s="3"/>
-      <c r="D196" s="3"/>
-      <c r="E196" s="3"/>
-      <c r="F196" s="3"/>
+      <c r="A196" s="4"/>
+      <c r="B196" s="4"/>
+      <c r="C196" s="4"/>
+      <c r="D196" s="4"/>
+      <c r="E196" s="4"/>
+      <c r="F196" s="4"/>
       <c r="G196" s="1"/>
       <c r="H196" s="1"/>
     </row>
     <row r="197" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A197" s="4"/>
-      <c r="B197" s="4"/>
-      <c r="C197" s="4"/>
-      <c r="D197" s="4"/>
-      <c r="E197" s="4"/>
-      <c r="F197" s="4"/>
+      <c r="A197" s="5"/>
+      <c r="B197" s="5"/>
+      <c r="C197" s="5"/>
+      <c r="D197" s="5"/>
+      <c r="E197" s="5"/>
+      <c r="F197" s="5"/>
       <c r="G197" s="1"/>
       <c r="H197" s="1"/>
     </row>
     <row r="198" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A198" s="8" t="s">
+      <c r="A198" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B198" s="7"/>
-      <c r="C198" s="2" t="s">
+      <c r="B198" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C198" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="D198" s="6" t="s">
+      <c r="D198" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="E198" s="5" t="s">
+      <c r="E198" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="F198" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G198" s="9" t="s">
+      <c r="F198" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G198" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="H198" s="9" t="s">
+      <c r="H198" s="2" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A199" s="3"/>
-      <c r="B199" s="3"/>
-      <c r="C199" s="3"/>
-      <c r="D199" s="3"/>
-      <c r="E199" s="3"/>
-      <c r="F199" s="3"/>
-      <c r="G199" s="9" t="s">
+      <c r="A199" s="4"/>
+      <c r="B199" s="4"/>
+      <c r="C199" s="4"/>
+      <c r="D199" s="4"/>
+      <c r="E199" s="4"/>
+      <c r="F199" s="4"/>
+      <c r="G199" s="2" t="s">
         <v>288</v>
       </c>
       <c r="H199" s="1"/>
     </row>
     <row r="200" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A200" s="3"/>
-      <c r="B200" s="3"/>
-      <c r="C200" s="3"/>
-      <c r="D200" s="3"/>
-      <c r="E200" s="3"/>
-      <c r="F200" s="3"/>
-      <c r="G200" s="9" t="s">
+      <c r="A200" s="4"/>
+      <c r="B200" s="4"/>
+      <c r="C200" s="4"/>
+      <c r="D200" s="4"/>
+      <c r="E200" s="4"/>
+      <c r="F200" s="4"/>
+      <c r="G200" s="2" t="s">
         <v>289</v>
       </c>
       <c r="H200" s="1"/>
     </row>
     <row r="201" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A201" s="4"/>
-      <c r="B201" s="4"/>
-      <c r="C201" s="4"/>
-      <c r="D201" s="4"/>
-      <c r="E201" s="4"/>
-      <c r="F201" s="4"/>
-      <c r="G201" s="9" t="s">
+      <c r="A201" s="5"/>
+      <c r="B201" s="5"/>
+      <c r="C201" s="5"/>
+      <c r="D201" s="5"/>
+      <c r="E201" s="5"/>
+      <c r="F201" s="5"/>
+      <c r="G201" s="2" t="s">
         <v>282</v>
       </c>
       <c r="H201" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="300">
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="A98:A101"/>
     <mergeCell ref="C14:C17"/>
     <mergeCell ref="B66:B69"/>
     <mergeCell ref="C98:C101"/>
@@ -4141,7 +4242,9 @@
     <mergeCell ref="A158:A161"/>
     <mergeCell ref="B34:B37"/>
     <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="B154:B157"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="E62:E65"/>
     <mergeCell ref="F50:F53"/>
     <mergeCell ref="F30:F33"/>
     <mergeCell ref="A54:A57"/>
@@ -4163,13 +4266,6 @@
     <mergeCell ref="E94:E97"/>
     <mergeCell ref="E90:E93"/>
     <mergeCell ref="F110:F113"/>
-    <mergeCell ref="D150:D153"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="F94:F97"/>
-    <mergeCell ref="B158:B161"/>
-    <mergeCell ref="D78:D81"/>
     <mergeCell ref="F98:F101"/>
     <mergeCell ref="C86:C89"/>
     <mergeCell ref="F82:F85"/>
@@ -4179,6 +4275,7 @@
     <mergeCell ref="C138:C141"/>
     <mergeCell ref="B74:B77"/>
     <mergeCell ref="F150:F153"/>
+    <mergeCell ref="D150:D153"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="C2:C5"/>
     <mergeCell ref="B6:B9"/>
@@ -4347,9 +4444,6 @@
     <mergeCell ref="E146:E149"/>
     <mergeCell ref="A58:A61"/>
     <mergeCell ref="F166:F169"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="B138:B141"/>
-    <mergeCell ref="E134:E137"/>
     <mergeCell ref="A170:A173"/>
     <mergeCell ref="D22:D25"/>
     <mergeCell ref="A70:A73"/>
@@ -4371,9 +4465,9 @@
     <mergeCell ref="F42:F45"/>
     <mergeCell ref="B118:B121"/>
     <mergeCell ref="E154:E157"/>
-    <mergeCell ref="B154:B157"/>
-    <mergeCell ref="C174:C177"/>
-    <mergeCell ref="F170:F173"/>
+    <mergeCell ref="F94:F97"/>
+    <mergeCell ref="B158:B161"/>
+    <mergeCell ref="D78:D81"/>
     <mergeCell ref="D6:D9"/>
     <mergeCell ref="D190:D193"/>
     <mergeCell ref="B86:B89"/>
@@ -4396,8 +4490,8 @@
     <mergeCell ref="D134:D137"/>
     <mergeCell ref="D74:D77"/>
     <mergeCell ref="C6:C9"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="B138:B141"/>
     <mergeCell ref="D194:D197"/>
     <mergeCell ref="F134:F137"/>
     <mergeCell ref="A198:A201"/>
@@ -4419,6 +4513,9 @@
     <mergeCell ref="C190:C193"/>
     <mergeCell ref="B114:B117"/>
     <mergeCell ref="D114:D117"/>
+    <mergeCell ref="C174:C177"/>
+    <mergeCell ref="F170:F173"/>
+    <mergeCell ref="E134:E137"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Excel after corrections of translations and with final corrections
</commit_message>
<xml_diff>
--- a/IT23681842-Assignment 1 - Test cases.xlsx
+++ b/IT23681842-Assignment 1 - Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SLIIT\3rd Year\1st Semester\ITPM\ITPM Assignment IT23681842\IT23681842\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46FE1579-FD1D-4722-87FE-8B1C00FB262D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1952C514-97AF-41B1-B606-786BB050C29C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -136,9 +136,6 @@
     <t>api ilaga mase 10 wenid wadihiti niwasekt kaama beema argena ymu enam</t>
   </si>
   <si>
-    <t>අපි ඊලග මාසේ 10 වෙනිදා වැඩිහිටි නිවාසෙකට කෑම බීම අරගෙන යමු එනම්</t>
-  </si>
-  <si>
     <t>හෙට හව්ස් 5 වෙද්දි වලි load 5ක් පන්නිපිටියට එවන්ව කිව්වා</t>
   </si>
   <si>
@@ -418,51 +415,33 @@
     <t>ඒ shoe එක koko වලින් ගන්නවනම් rs 8000ක් වෙනවා, එක ලාභයි.</t>
   </si>
   <si>
-    <t>ඒ shoe එක කොකෝ වලින් ගන්නවනම් rs 8000ක් වෙනවා, එක ලාභයි.</t>
-  </si>
-  <si>
     <t>mt heta ude 8 ta hire ekak ynna thiyenawa bibile ta</t>
   </si>
   <si>
     <t>මට හෙට උදේ 8 ට හයර් එකක් යන්න තියෙනවා බිබිල ට.</t>
   </si>
   <si>
-    <t>මට හෙට උදේ 8 ට හිර‍ෙ එකක් යන්න තියෙනවා බිබිලේට</t>
-  </si>
-  <si>
     <t>anidda raa 8 ta one gall face eke function ekak thiyenawa eka blnna ymuda?</t>
   </si>
   <si>
     <t>අනිද්දා රෑ 8ට one gall face එකේ function එකක් තියෙනවා ඒක බලන්න යමුද?</t>
   </si>
   <si>
-    <t>අනිද්දා රෑ 8ට වන් ගොල් ෆේස් එකේ function එකක් තියෙනවා  ඒක බලන්න යමුද?</t>
-  </si>
-  <si>
     <t>2026-05-10 test ekak thiyenawa eka byod widiht thiyenne</t>
   </si>
   <si>
     <t>2026-05-10  test එකක් තියෙනවා ඒක BYOD විදිහට තියෙන්නේ.</t>
   </si>
   <si>
-    <t>2026-05-10  test එකක් තියෙනවා ඒක බයෝඩ් විදිහට තියෙන්නේ.</t>
-  </si>
-  <si>
     <t>march 20 thibba event ekt support ek dunnt oyl hamotama thnx hode</t>
   </si>
   <si>
     <t>මාර්තු 20 තිබ්බ event එකට support එක දුන්නට ඔයාලා හැමෝටම thnx හොඳේ.</t>
   </si>
   <si>
-    <t>මාර්තු 20 තිබ්බ event එකට support එක දුන්නට ඔයාලා හැමෝටම ත්න්ක්ස් හොඳේ.</t>
-  </si>
-  <si>
     <t>XXL shirt ekak koko walin gannawanan godak mila aduwata gnna puluwan, eka godak labai koko haraha gnna eka</t>
   </si>
   <si>
-    <t>XXL shirt එකක් කොකෝ වලින් ගන්නවනම් ගොඩක් මිල අඩුවට ගන්න පුළුවන්, එක ගොඩක් ලාභයි කොකෝ හරහා ගන්න එක.</t>
-  </si>
-  <si>
     <t>XXL shirt එකක් koko වලින් ගන්නවනම් ගොඩක් මිල අඩුවට ගන්න පුළුවන්, එක ගොඩක් ලාභයි koko හරහා ගන්න එක.</t>
   </si>
   <si>
@@ -470,9 +449,6 @@
   </si>
   <si>
     <t>400 km වගේ හයර් එකක් තමයි ඒ හයර් එක, ඒක ගියානම් high profit එකක් ගන්න තිබ්බ.</t>
-  </si>
-  <si>
-    <t>400 ක්ම් වගේ හිරේ එකක් තමයි ඒ හිරේ එක, ඒක ගියානම් high profit එකක් ගන්න තිබ්බ.</t>
   </si>
   <si>
     <t>mage mail eka isinduduldara05@gmail.com, oyala ewana msg okkoma me mail ekata ewanna</t>
@@ -482,23 +458,13 @@
 , ඔයාලා එවන message ඔක්කොම මේ mail එකට එවන්න</t>
   </si>
   <si>
-    <t>මගේ mail එක isinduduldara05@gmail.කොම්
-, ඔයාලා එවන message ඔක්කොම මේ mail එකට එවන්න</t>
-  </si>
-  <si>
     <t>api hamoma ekathu wela project eka complete kara ehenam, hamotama godak thnx</t>
   </si>
   <si>
     <t>අපි හැමෝම එකතු වෙලා project එක complete කරා එහෙනම්, හැමෝටම ගොඩක් thnx</t>
   </si>
   <si>
-    <t>අපි හැමෝම එකතු වෙලා project එක complete කරා එහෙනම්, හැමෝටම ගොඩක් ත්න්ක්ස්</t>
-  </si>
-  <si>
     <t>oyalata edineda news danaganna https://www.lankadeepa.lk me link eken gihilla wisthara blnna</t>
-  </si>
-  <si>
-    <t>ඔයාලට එදිනෙදා news දැනගන්න https://www.lankadeepa.ල්ක් මේ ලින්ක් එකෙං ගිහිල්ලා විස්තර බලන්න</t>
   </si>
   <si>
     <t>ඔයාලට එදිනෙදා news දැනගන්න https://www.lankadeepa.lk මේ ලින්ක් එකෙං ගිහිල්ලා විස්තර බලන්න</t>
@@ -511,16 +477,9 @@
 මම check කරලා බලන්නම්</t>
   </si>
   <si>
-    <t>මට mail එකක් එවන්න isinduduldara05@gmail.කොම්
-මම check කරලා බලන්නම්</t>
-  </si>
-  <si>
     <t>mama oyalawa iye dakka  one gall face ekedi 🙃😎🤩</t>
   </si>
   <si>
-    <t xml:space="preserve">මම ඔයාලව ඊයේ දැක්කා one gall face එකේදී □□□ </t>
-  </si>
-  <si>
     <t>මම ඔයාලව ඊයේ දැක්කා one gall face එකේදී 🙃😎🤩</t>
   </si>
   <si>
@@ -533,22 +492,13 @@
     <t>ඔයාලගේ ගෙවල් තියෙන්නේ අරවල පාරේ නේද? □</t>
   </si>
   <si>
-    <t>oya heta 7.30pm ta zoom ekata join wenwda nathnm api time ek change krmu bn mokadda plan eka</t>
-  </si>
-  <si>
     <t>ඔයා හෙට 7.30pm ට Zoom එකට join වෙනවද නැත්නම් අපි time එක change කරමු බන් මොකද්ද plan එක</t>
   </si>
   <si>
-    <t>ඔය හෙට 7.30pm ට Zoom එකට join වෙනවද නැත්නම් අපි time එක change කරමු බන් මොකද්ද plan එක</t>
-  </si>
-  <si>
     <t>mama tiranya fashion eken gaththa dress eka size ek hariyata fit wenne na wage, oya balala exchange krnna puluwnda kiyala ahanna 🥹</t>
   </si>
   <si>
     <t>මම Tiranya Fashion එකෙන් ගත්ත dress එක size එක හරියට fit වෙන්නේ නැ වගේ ඔයා බලලා exchange කරන්න පුළුවන්ද කියලා අහන්න</t>
-  </si>
-  <si>
-    <t>මම ටිරනය Fashion එකෙන් ගත්ත dress එක size එක හරිට fit වෙන්නේ නැ වගේ ඔයා බලලා exchange කරන්න පුළුවන්ද කියලා අහන්න</t>
   </si>
   <si>
     <t xml:space="preserve">අයෝඩයට කියන්න පුළුවන්නම් අදම මට Call එකක් දෙන්න කියලා
@@ -598,60 +548,15 @@
     <t>වලි ලෝඩ් එකක් rs 16800 ක් වෙනවා</t>
   </si>
   <si>
-    <t>watch එක කැඩිලා නිසා අත් පලුවට ගිහිල්ලා</t>
-  </si>
-  <si>
-    <t>wifi එකට signal නෑ මේ දවස්වල වහින් නිසඩ කොහෙද</t>
-  </si>
-  <si>
-    <t>just try, try එකක් දීලා බලන්න, if u are unable to complete, මට කියන්න මම  එතකොට වෙන විදිහක අභයසයක් කල්පනා කරලා බලන්නම්</t>
-  </si>
-  <si>
     <t>if you are coming please tell me because, මට මොනා හරි හදන්න පුළුවන් ඔය වෙනුවෙන් dinner එකට</t>
   </si>
   <si>
-    <t>මේ lap එකේ power case එකක් තියෙනවා කියල තමා customer අපිට් කිව්වෙ</t>
-  </si>
-  <si>
-    <t>office එකෙන් notice එකක් දාලා තිබ්බ අද zoom meeting එක හැමෝටම් compulsory කියලා, ඒකෙදි year plan එක ග්න් කතා කරනවා කියලත් කිව්වා</t>
-  </si>
-  <si>
-    <t>නිපුන කියන්නේ විශේෂ අධ්‍පනය යටතේ ඉගෙන ගන්න ලමයෙක් නේද? අපිට පුලුවන් එයාටත් උදව්වක් කරන්න</t>
-  </si>
-  <si>
-    <t>අම්මා කිව්වා තැබිලි ගහෙන් ගෙඩි 5ක් කඩාගෙන පන්ස්ට ගෙනියන්න කියලා</t>
-  </si>
-  <si>
-    <t>ඒක පාතමික් විදුහලක්ද ? හැබැයි අපිට ඒ ස්කෝලේටත් උදව්වක් කරගෙනම් යන්න පුළුවන්…</t>
-  </si>
-  <si>
-    <t>අනේ ! අරව්වල පාරේ වාහන තුනක් එකට හැප්පිලා දෙන්නෙක් මැරිලලු... පව් එයාලා...</t>
-  </si>
-  <si>
-    <t xml:space="preserve">නෑ නෑ එයා කියපු විදිහට වාහනේ වැඩේ සෑහෙන් කල් යන් වැඩක් කිව්වා  </t>
-  </si>
-  <si>
     <t xml:space="preserve">නෑ නෑ එයා කියපු විදිහට වාහනේ වැඩේ සෑහෙන කල් යන වැඩක් කිව්වා  </t>
   </si>
   <si>
-    <t>තුන්වෙනි උපන්දිනය සමරන් පුංචි පුතාට් සුබම සුබ උපන්දිනයක් වේවා !</t>
-  </si>
-  <si>
-    <t>ආයුභෝවන් සර් ! ඔයාට ටික වෙලාවක් අමතුමේ රෑදී ඉන්න වෙනවා</t>
-  </si>
-  <si>
-    <t>ඔය හෙට උදේ 8 වෙන්කොට කොළඹ කොටුවට යන්න</t>
-  </si>
-  <si>
     <t>oya labna weekend eketh gdra yanne nathuwa innada hdnne ?</t>
   </si>
   <si>
-    <t>ඔය ලබන weekend එකෙත් ගදර යන්නේ නැතුව ඉන්නද හදන්නේ ?</t>
-  </si>
-  <si>
-    <t>අද පාඩම හරියට තේරුනද නද්ද ඉසිඳු ?</t>
-  </si>
-  <si>
     <t>Singlish input types covered</t>
   </si>
   <si>
@@ -902,6 +807,99 @@
   </si>
   <si>
     <t>S</t>
+  </si>
+  <si>
+    <t>අද පාඩම හරියට තේරුනාද නද්ද ඉසිඳු ?</t>
+  </si>
+  <si>
+    <t>ඔය ලබන weekend එකෙත් ගෙදර යන්නේ නැතුව ඉන්නද හදන්නේ ?</t>
+  </si>
+  <si>
+    <t>ඔයා හෙට උදේ 8 වෙන්කොට කොලබ කොටුවට යන්න</t>
+  </si>
+  <si>
+    <t>ආයුභෝවන් sir ! ඔයාට ටික වෙලාවක් අමතුමේ රෑදී ඉන්න වෙනවා</t>
+  </si>
+  <si>
+    <t>තුන්වෙනි උපන්දිනය සමර්න් පුංචි පුතාට් සුබම සුබ උපන්දිනයක් වේවා !</t>
+  </si>
+  <si>
+    <t>අපි ඊලග මාසේ 10 වෙනිදා වැඩිහිටි නිවාසෙකට කෑම බීම අරගෙන යමු එ්නම්</t>
+  </si>
+  <si>
+    <t>නෑ නෑ ඇයි කියපු විදිහට වාහනේ වැඩේ සහෙන් කල් යමු වැඩක් කිව්වා</t>
+  </si>
+  <si>
+    <t>අනේ ! අරව්වල පාරේ වාහන තුන්ක් එකට හප්පිලා දෙන්නෙක් මැරිලාලු... පව් එයාලා...</t>
+  </si>
+  <si>
+    <t>ඒක ප්රාත්මික විදුහලක්ද ? හැබැයි අපිට ඒ ස්කෝලේටත් උදව්වක් කරගෙනම් යන්න පුළුවන්...</t>
+  </si>
+  <si>
+    <t>අම්මා කිව්වා තැබිලි ගහෙන් ගෙඩි 5ක් කඩෙන් පින්ස්ලාට ගෙනියන්න කියලා</t>
+  </si>
+  <si>
+    <t>නිපුණ කියන්නේ විශේෂ අද්යාපනය යටතෙ ඉගෙන ගන්න ල්ම්යෙක් නේද? අපිට පුළුවන් එයාටත් උදව්වක් කරන්න</t>
+  </si>
+  <si>
+    <t>office එකෙන් notice එකක් දාලා තිබ්බ අද zoom meeting එක හැමෝටම compulsory කියලා, ඒකෙදි year plan එක ගැන කතා කරනවා කියලාත් කිව්වා</t>
+  </si>
+  <si>
+    <t>මේ lap එකේ power case එකක් තියෙනවා කියලා තමයි customer අපිටත් කිව්වේ</t>
+  </si>
+  <si>
+    <t>just try, try එකක් දීලා බලන්න, if u are unable to complete, මට කියන්න මන් එතකොට වෙන විදිහක් අබ්යාසයක් කල්පනා කරලා බලන්නම්</t>
+  </si>
+  <si>
+    <t>wifi එකට signal නෑ මේ දවස්වල වහින් නිසාද කොහේද</t>
+  </si>
+  <si>
+    <t>watch එක කැඩිලා නිසා අත් ප්ලුවට ගිහිල්ලා</t>
+  </si>
+  <si>
+    <t>ඒ shoe එක කොකෝ වලින් ගන්නවනං Rs 8000ක් වෙනවා , ඒක ලාබය්</t>
+  </si>
+  <si>
+    <t>මට හෙට උදේ 8 ට හිරේ එකක් යන්න තියෙනවා බිබිලේ ට</t>
+  </si>
+  <si>
+    <t>අනිද්දා රා 8 ට one gall face එකේ function එකක් තියෙනවා ඒක බලන්න යමුද?</t>
+  </si>
+  <si>
+    <t>2026-05-10 ටෙස්ට් එකක් තියෙනවා ඒක බයෝඩ් විදිහට තියෙන්නේ</t>
+  </si>
+  <si>
+    <t>මාර්තු 20 තිබ්බ event එකට support එක දුන්නට ඔයාලා හැමෝටම තෑන්ක්ස් හොදේ</t>
+  </si>
+  <si>
+    <t>XXL ෂර්ට් එකක් කොකෝ වලින් ගන්නවනං ගොඩක් මිල අඩුවට ගන්න පුලුවන්, ඒක ගොඩක් ලයිකා කෝකෝ හරහා ගන්න එක</t>
+  </si>
+  <si>
+    <t>400 km වගේ හිරේ එකක් තමා ඒ හිරේ එක, ඒක ගියානං high profit එකක් ගන්න තිබ්බා</t>
+  </si>
+  <si>
+    <t>මගේ mail එක ඉසින්දුදුල්දර05@gmail.කොම්, ඔයාලා එවන msg ඔක්කොම මේ mail එකට එවන්න</t>
+  </si>
+  <si>
+    <t>අපි හැමෝම එකතු වෙලා project එක complete කර එහෙනම්, හැමෝටම ගොඩක් තෑන්ක්ස්</t>
+  </si>
+  <si>
+    <t>ඔයාලට එදිනෙදා news දානගන්න https://www.ලංකාදීප.ලැක් මේ link එකෙන් ගිහිල්ලා විස්තර බලන්න</t>
+  </si>
+  <si>
+    <t>මට mail එකක් එවන්න ඉසින්දුදුල්දර05@gmail.කොම් මම චෙක් කරලා බලන්නම්</t>
+  </si>
+  <si>
+    <t>මම ඔයාලව ඊයේ දැක්කා ඕනේ gall face එකේදී 😎</t>
+  </si>
+  <si>
+    <t>ඔය හෙට 7.30pm ට zoom එකට join වෙනවද නැත්නම් අපි time එක change කරමු බන් මොකද්ද plan එක</t>
+  </si>
+  <si>
+    <t>oy heta 7.30pm ta zoom ekata join wenwda nathnm api time ek change krmu bn mokadda plan eka</t>
+  </si>
+  <si>
+    <t>මම ටි්රන්ය ෆෝඩ් එකෙන් ගත්ත dress එක size එක හරියට fit වෙන්නේ නෑ වගේ, ඔයා බලලා exchange කරන්න පුළුවන්ද කියලා අහන්න</t>
   </si>
 </sst>
 </file>
@@ -1344,10 +1342,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>208</v>
+        <v>177</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>209</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1355,7 +1353,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>291</v>
+        <v>260</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>8</v>
@@ -1364,16 +1362,16 @@
         <v>9</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>207</v>
+        <v>261</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>211</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1414,22 +1412,22 @@
         <v>7</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>206</v>
+        <v>262</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>213</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1440,7 +1438,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="2" t="s">
-        <v>212</v>
+        <v>181</v>
       </c>
       <c r="H7" s="1"/>
     </row>
@@ -1478,16 +1476,16 @@
         <v>15</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>204</v>
+        <v>263</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>214</v>
+        <v>183</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>216</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1498,7 +1496,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="2" t="s">
-        <v>215</v>
+        <v>184</v>
       </c>
       <c r="H11" s="1"/>
     </row>
@@ -1542,10 +1540,10 @@
         <v>10</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>217</v>
+        <v>186</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>218</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1556,7 +1554,7 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="2" t="s">
-        <v>215</v>
+        <v>184</v>
       </c>
       <c r="H15" s="1"/>
     </row>
@@ -1594,16 +1592,16 @@
         <v>22</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>203</v>
+        <v>264</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>219</v>
+        <v>188</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>221</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1614,7 +1612,7 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="2" t="s">
-        <v>220</v>
+        <v>189</v>
       </c>
       <c r="H19" s="1"/>
     </row>
@@ -1652,16 +1650,16 @@
         <v>25</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>202</v>
+        <v>265</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>219</v>
+        <v>188</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>222</v>
+        <v>191</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1708,16 +1706,16 @@
         <v>28</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>223</v>
+        <v>192</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>224</v>
+        <v>193</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1728,7 +1726,7 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="2" t="s">
-        <v>212</v>
+        <v>181</v>
       </c>
       <c r="H27" s="1"/>
     </row>
@@ -1772,10 +1770,10 @@
         <v>10</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>225</v>
+        <v>194</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>226</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1786,7 +1784,7 @@
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="2" t="s">
-        <v>212</v>
+        <v>181</v>
       </c>
       <c r="H31" s="1"/>
     </row>
@@ -1824,16 +1822,16 @@
         <v>35</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>214</v>
+        <v>183</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>227</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1844,7 +1842,7 @@
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="2" t="s">
-        <v>225</v>
+        <v>194</v>
       </c>
       <c r="H35" s="1"/>
     </row>
@@ -1879,19 +1877,19 @@
         <v>37</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>38</v>
+        <v>266</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>228</v>
+        <v>197</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>229</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1926,28 +1924,28 @@
     </row>
     <row r="42" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>201</v>
+        <v>175</v>
       </c>
       <c r="E42" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H42" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1982,28 +1980,28 @@
     </row>
     <row r="46" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>217</v>
+        <v>186</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>232</v>
+        <v>201</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2038,28 +2036,28 @@
     </row>
     <row r="50" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C50" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D50" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D50" s="3" t="s">
-        <v>84</v>
-      </c>
       <c r="E50" s="9" t="s">
-        <v>199</v>
+        <v>268</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>220</v>
+        <v>189</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>234</v>
+        <v>203</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2070,7 +2068,7 @@
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="2" t="s">
-        <v>233</v>
+        <v>202</v>
       </c>
       <c r="H51" s="1"/>
     </row>
@@ -2096,28 +2094,28 @@
     </row>
     <row r="54" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C54" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D54" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D54" s="3" t="s">
-        <v>86</v>
-      </c>
       <c r="E54" s="9" t="s">
-        <v>198</v>
+        <v>269</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>235</v>
+        <v>204</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2152,28 +2150,28 @@
     </row>
     <row r="58" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C58" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D58" s="3" t="s">
-        <v>88</v>
-      </c>
       <c r="E58" s="9" t="s">
-        <v>197</v>
+        <v>270</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>237</v>
+        <v>206</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2184,7 +2182,7 @@
       <c r="E59" s="4"/>
       <c r="F59" s="4"/>
       <c r="G59" s="2" t="s">
-        <v>217</v>
+        <v>186</v>
       </c>
       <c r="H59" s="1"/>
     </row>
@@ -2210,28 +2208,28 @@
     </row>
     <row r="62" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>196</v>
+        <v>271</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>238</v>
+        <v>207</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2266,28 +2264,28 @@
     </row>
     <row r="66" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C66" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D66" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D66" s="3" t="s">
-        <v>92</v>
-      </c>
       <c r="E66" s="9" t="s">
-        <v>195</v>
+        <v>272</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>239</v>
+        <v>208</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>241</v>
+        <v>210</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2298,7 +2296,7 @@
       <c r="E67" s="4"/>
       <c r="F67" s="4"/>
       <c r="G67" s="2" t="s">
-        <v>240</v>
+        <v>209</v>
       </c>
       <c r="H67" s="1"/>
     </row>
@@ -2324,28 +2322,28 @@
     </row>
     <row r="70" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C70" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D70" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D70" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="E70" s="9" t="s">
-        <v>194</v>
+        <v>273</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>242</v>
+        <v>211</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>243</v>
+        <v>212</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2380,28 +2378,28 @@
     </row>
     <row r="74" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C74" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="D74" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D74" s="3" t="s">
-        <v>96</v>
-      </c>
       <c r="E74" s="9" t="s">
-        <v>193</v>
+        <v>174</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>244</v>
+        <v>213</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>245</v>
+        <v>214</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2436,28 +2434,28 @@
     </row>
     <row r="78" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B78" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C78" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D78" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="D78" s="3" t="s">
-        <v>98</v>
-      </c>
       <c r="E78" s="9" t="s">
-        <v>192</v>
+        <v>274</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>244</v>
+        <v>213</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>246</v>
+        <v>215</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2492,28 +2490,28 @@
     </row>
     <row r="82" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B82" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C82" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D82" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D82" s="3" t="s">
-        <v>100</v>
-      </c>
       <c r="E82" s="9" t="s">
-        <v>191</v>
+        <v>275</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>242</v>
+        <v>211</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>247</v>
+        <v>216</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2548,28 +2546,28 @@
     </row>
     <row r="86" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B86" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C86" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="D86" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D86" s="3" t="s">
-        <v>102</v>
-      </c>
       <c r="E86" s="9" t="s">
-        <v>190</v>
+        <v>276</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>212</v>
+        <v>181</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>248</v>
+        <v>217</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2604,28 +2602,28 @@
     </row>
     <row r="90" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B90" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C90" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D90" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D90" s="3" t="s">
-        <v>108</v>
-      </c>
       <c r="E90" s="9" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>239</v>
+        <v>208</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>249</v>
+        <v>218</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2660,28 +2658,28 @@
     </row>
     <row r="94" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B94" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C94" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="D94" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="D94" s="3" t="s">
-        <v>110</v>
-      </c>
       <c r="E94" s="9" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>239</v>
+        <v>208</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>250</v>
+        <v>219</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2716,28 +2714,28 @@
     </row>
     <row r="98" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B98" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C98" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="D98" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D98" s="3" t="s">
-        <v>104</v>
-      </c>
       <c r="E98" s="9" t="s">
-        <v>178</v>
+        <v>162</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>251</v>
+        <v>220</v>
       </c>
       <c r="H98" s="2" t="s">
-        <v>252</v>
+        <v>221</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2772,28 +2770,28 @@
     </row>
     <row r="102" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B102" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C102" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D102" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="D102" s="3" t="s">
-        <v>106</v>
-      </c>
       <c r="E102" s="9" t="s">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>253</v>
+        <v>222</v>
       </c>
       <c r="H102" s="2" t="s">
-        <v>255</v>
+        <v>224</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2804,7 +2802,7 @@
       <c r="E103" s="4"/>
       <c r="F103" s="4"/>
       <c r="G103" s="2" t="s">
-        <v>254</v>
+        <v>223</v>
       </c>
       <c r="H103" s="1"/>
     </row>
@@ -2830,28 +2828,28 @@
     </row>
     <row r="106" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B106" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C106" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D106" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D106" s="3" t="s">
-        <v>112</v>
-      </c>
       <c r="E106" s="9" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>215</v>
+        <v>184</v>
       </c>
       <c r="H106" s="2" t="s">
-        <v>257</v>
+        <v>226</v>
       </c>
     </row>
     <row r="107" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2862,7 +2860,7 @@
       <c r="E107" s="4"/>
       <c r="F107" s="4"/>
       <c r="G107" s="2" t="s">
-        <v>256</v>
+        <v>225</v>
       </c>
       <c r="H107" s="1"/>
     </row>
@@ -2888,28 +2886,28 @@
     </row>
     <row r="110" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B110" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C110" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D110" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D110" s="3" t="s">
-        <v>114</v>
-      </c>
       <c r="E110" s="9" t="s">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>212</v>
+        <v>181</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>258</v>
+        <v>227</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2944,28 +2942,28 @@
     </row>
     <row r="114" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B114" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C114" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D114" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D114" s="3" t="s">
-        <v>116</v>
-      </c>
       <c r="E114" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="F114" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G114" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F114" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G114" s="2" t="s">
-        <v>215</v>
-      </c>
       <c r="H114" s="2" t="s">
-        <v>259</v>
+        <v>228</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2976,7 +2974,7 @@
       <c r="E115" s="4"/>
       <c r="F115" s="4"/>
       <c r="G115" s="2" t="s">
-        <v>256</v>
+        <v>225</v>
       </c>
       <c r="H115" s="1"/>
     </row>
@@ -3002,28 +3000,28 @@
     </row>
     <row r="118" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B118" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C118" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="D118" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D118" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="E118" s="9" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>215</v>
+        <v>184</v>
       </c>
       <c r="H118" s="2" t="s">
-        <v>260</v>
+        <v>229</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3034,7 +3032,7 @@
       <c r="E119" s="4"/>
       <c r="F119" s="4"/>
       <c r="G119" s="2" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="H119" s="1"/>
     </row>
@@ -3060,28 +3058,28 @@
     </row>
     <row r="122" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B122" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C122" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="D122" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D122" s="3" t="s">
-        <v>121</v>
-      </c>
       <c r="E122" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G122" s="2" t="s">
-        <v>261</v>
+        <v>230</v>
       </c>
       <c r="H122" s="2" t="s">
-        <v>262</v>
+        <v>231</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3116,28 +3114,28 @@
     </row>
     <row r="126" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B126" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C126" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="D126" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="D126" s="3" t="s">
-        <v>123</v>
-      </c>
       <c r="E126" s="9" t="s">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="F126" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>215</v>
+        <v>184</v>
       </c>
       <c r="H126" s="2" t="s">
-        <v>263</v>
+        <v>232</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3172,28 +3170,28 @@
     </row>
     <row r="130" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B130" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C130" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D130" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D130" s="3" t="s">
-        <v>125</v>
-      </c>
       <c r="E130" s="9" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="F130" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="H130" s="2" t="s">
-        <v>264</v>
+        <v>233</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3228,28 +3226,28 @@
     </row>
     <row r="134" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B134" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C134" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D134" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="D134" s="3" t="s">
-        <v>127</v>
-      </c>
       <c r="E134" s="9" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="F134" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G134" s="2" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="H134" s="2" t="s">
-        <v>266</v>
+        <v>235</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3260,7 +3258,7 @@
       <c r="E135" s="4"/>
       <c r="F135" s="4"/>
       <c r="G135" s="2" t="s">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="H135" s="1"/>
     </row>
@@ -3272,7 +3270,7 @@
       <c r="E136" s="4"/>
       <c r="F136" s="4"/>
       <c r="G136" s="2" t="s">
-        <v>265</v>
+        <v>234</v>
       </c>
       <c r="H136" s="1"/>
     </row>
@@ -3288,28 +3286,28 @@
     </row>
     <row r="138" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B138" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C138" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D138" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="D138" s="3" t="s">
-        <v>129</v>
-      </c>
       <c r="E138" s="9" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="F138" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G138" s="2" t="s">
-        <v>267</v>
+        <v>236</v>
       </c>
       <c r="H138" s="2" t="s">
-        <v>268</v>
+        <v>237</v>
       </c>
     </row>
     <row r="139" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3320,7 +3318,7 @@
       <c r="E139" s="4"/>
       <c r="F139" s="4"/>
       <c r="G139" s="2" t="s">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="H139" s="1"/>
     </row>
@@ -3346,28 +3344,28 @@
     </row>
     <row r="142" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B142" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C142" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="D142" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="D142" s="3" t="s">
-        <v>131</v>
-      </c>
       <c r="E142" s="9" t="s">
-        <v>132</v>
+        <v>277</v>
       </c>
       <c r="F142" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G142" s="2" t="s">
-        <v>267</v>
+        <v>236</v>
       </c>
       <c r="H142" s="2" t="s">
-        <v>269</v>
+        <v>238</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3378,7 +3376,7 @@
       <c r="E143" s="4"/>
       <c r="F143" s="4"/>
       <c r="G143" s="2" t="s">
-        <v>256</v>
+        <v>225</v>
       </c>
       <c r="H143" s="1"/>
     </row>
@@ -3404,28 +3402,28 @@
     </row>
     <row r="146" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B146" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C146" s="8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E146" s="9" t="s">
-        <v>135</v>
+        <v>278</v>
       </c>
       <c r="F146" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G146" s="2" t="s">
-        <v>214</v>
+        <v>183</v>
       </c>
       <c r="H146" s="2" t="s">
-        <v>271</v>
+        <v>240</v>
       </c>
     </row>
     <row r="147" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3436,7 +3434,7 @@
       <c r="E147" s="4"/>
       <c r="F147" s="4"/>
       <c r="G147" s="2" t="s">
-        <v>270</v>
+        <v>239</v>
       </c>
       <c r="H147" s="1"/>
     </row>
@@ -3462,28 +3460,28 @@
     </row>
     <row r="150" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B150" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E150" s="9" t="s">
-        <v>138</v>
+        <v>279</v>
       </c>
       <c r="F150" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G150" s="2" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="H150" s="2" t="s">
-        <v>272</v>
+        <v>241</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3494,7 +3492,7 @@
       <c r="E151" s="4"/>
       <c r="F151" s="4"/>
       <c r="G151" s="2" t="s">
-        <v>214</v>
+        <v>183</v>
       </c>
       <c r="H151" s="1"/>
     </row>
@@ -3506,7 +3504,7 @@
       <c r="E152" s="4"/>
       <c r="F152" s="4"/>
       <c r="G152" s="2" t="s">
-        <v>270</v>
+        <v>239</v>
       </c>
       <c r="H152" s="1"/>
     </row>
@@ -3522,28 +3520,28 @@
     </row>
     <row r="154" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B154" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C154" s="8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E154" s="9" t="s">
-        <v>141</v>
+        <v>280</v>
       </c>
       <c r="F154" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G154" s="2" t="s">
-        <v>228</v>
+        <v>197</v>
       </c>
       <c r="H154" s="2" t="s">
-        <v>273</v>
+        <v>242</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3554,7 +3552,7 @@
       <c r="E155" s="4"/>
       <c r="F155" s="4"/>
       <c r="G155" s="2" t="s">
-        <v>240</v>
+        <v>209</v>
       </c>
       <c r="H155" s="1"/>
     </row>
@@ -3580,28 +3578,28 @@
     </row>
     <row r="158" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B158" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C158" s="8" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E158" s="9" t="s">
-        <v>144</v>
+        <v>281</v>
       </c>
       <c r="F158" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G158" s="2" t="s">
-        <v>228</v>
+        <v>197</v>
       </c>
       <c r="H158" s="2" t="s">
-        <v>274</v>
+        <v>243</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3612,7 +3610,7 @@
       <c r="E159" s="4"/>
       <c r="F159" s="4"/>
       <c r="G159" s="2" t="s">
-        <v>233</v>
+        <v>202</v>
       </c>
       <c r="H159" s="1"/>
     </row>
@@ -3638,28 +3636,28 @@
     </row>
     <row r="162" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B162" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C162" s="8" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="E162" s="9" t="s">
-        <v>146</v>
+        <v>282</v>
       </c>
       <c r="F162" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G162" s="2" t="s">
-        <v>275</v>
+        <v>244</v>
       </c>
       <c r="H162" s="2" t="s">
-        <v>276</v>
+        <v>245</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3670,7 +3668,7 @@
       <c r="E163" s="4"/>
       <c r="F163" s="4"/>
       <c r="G163" s="2" t="s">
-        <v>256</v>
+        <v>225</v>
       </c>
       <c r="H163" s="1"/>
     </row>
@@ -3696,28 +3694,28 @@
     </row>
     <row r="166" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B166" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C166" s="8" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="E166" s="9" t="s">
-        <v>150</v>
+        <v>283</v>
       </c>
       <c r="F166" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G166" s="2" t="s">
-        <v>225</v>
+        <v>194</v>
       </c>
       <c r="H166" s="2" t="s">
-        <v>277</v>
+        <v>246</v>
       </c>
     </row>
     <row r="167" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3728,7 +3726,7 @@
       <c r="E167" s="4"/>
       <c r="F167" s="4"/>
       <c r="G167" s="2" t="s">
-        <v>256</v>
+        <v>225</v>
       </c>
       <c r="H167" s="1"/>
     </row>
@@ -3754,28 +3752,28 @@
     </row>
     <row r="170" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B170" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C170" s="8" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="E170" s="9" t="s">
-        <v>153</v>
+        <v>284</v>
       </c>
       <c r="F170" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G170" s="2" t="s">
-        <v>278</v>
+        <v>247</v>
       </c>
       <c r="H170" s="2" t="s">
-        <v>279</v>
+        <v>248</v>
       </c>
     </row>
     <row r="171" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3810,28 +3808,28 @@
     </row>
     <row r="174" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B174" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C174" s="8" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E174" s="9" t="s">
-        <v>156</v>
+        <v>285</v>
       </c>
       <c r="F174" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G174" s="2" t="s">
-        <v>256</v>
+        <v>225</v>
       </c>
       <c r="H174" s="2" t="s">
-        <v>280</v>
+        <v>249</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3842,7 +3840,7 @@
       <c r="E175" s="4"/>
       <c r="F175" s="4"/>
       <c r="G175" s="2" t="s">
-        <v>233</v>
+        <v>202</v>
       </c>
       <c r="H175" s="1"/>
     </row>
@@ -3868,28 +3866,28 @@
     </row>
     <row r="178" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B178" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C178" s="8" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E178" s="9" t="s">
-        <v>158</v>
+        <v>286</v>
       </c>
       <c r="F178" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G178" s="2" t="s">
-        <v>278</v>
+        <v>247</v>
       </c>
       <c r="H178" s="2" t="s">
-        <v>281</v>
+        <v>250</v>
       </c>
     </row>
     <row r="179" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3924,28 +3922,28 @@
     </row>
     <row r="182" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B182" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C182" s="8" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="D182" s="3" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="E182" s="9" t="s">
-        <v>162</v>
+        <v>287</v>
       </c>
       <c r="F182" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G182" s="2" t="s">
-        <v>278</v>
+        <v>247</v>
       </c>
       <c r="H182" s="2" t="s">
-        <v>279</v>
+        <v>248</v>
       </c>
     </row>
     <row r="183" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3980,28 +3978,28 @@
     </row>
     <row r="186" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B186" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C186" s="8" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="D186" s="3" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="E186" s="9" t="s">
-        <v>164</v>
+        <v>288</v>
       </c>
       <c r="F186" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G186" s="2" t="s">
-        <v>282</v>
+        <v>251</v>
       </c>
       <c r="H186" s="2" t="s">
-        <v>283</v>
+        <v>252</v>
       </c>
     </row>
     <row r="187" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4012,7 +4010,7 @@
       <c r="E187" s="4"/>
       <c r="F187" s="4"/>
       <c r="G187" s="2" t="s">
-        <v>270</v>
+        <v>239</v>
       </c>
       <c r="H187" s="1"/>
     </row>
@@ -4038,28 +4036,28 @@
     </row>
     <row r="190" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B190" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C190" s="8" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="D190" s="3" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="E190" s="9" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="F190" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G190" s="2" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="H190" s="2" t="s">
-        <v>284</v>
+        <v>253</v>
       </c>
     </row>
     <row r="191" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4070,7 +4068,7 @@
       <c r="E191" s="4"/>
       <c r="F191" s="4"/>
       <c r="G191" s="2" t="s">
-        <v>282</v>
+        <v>251</v>
       </c>
       <c r="H191" s="1"/>
     </row>
@@ -4096,28 +4094,28 @@
     </row>
     <row r="194" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B194" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C194" s="8" t="s">
-        <v>169</v>
+        <v>290</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="E194" s="9" t="s">
-        <v>171</v>
+        <v>289</v>
       </c>
       <c r="F194" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G194" s="2" t="s">
-        <v>214</v>
+        <v>183</v>
       </c>
       <c r="H194" s="2" t="s">
-        <v>286</v>
+        <v>255</v>
       </c>
     </row>
     <row r="195" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4128,7 +4126,7 @@
       <c r="E195" s="4"/>
       <c r="F195" s="4"/>
       <c r="G195" s="2" t="s">
-        <v>285</v>
+        <v>254</v>
       </c>
       <c r="H195" s="1"/>
     </row>
@@ -4154,28 +4152,28 @@
     </row>
     <row r="198" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B198" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C198" s="8" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="D198" s="3" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="E198" s="9" t="s">
-        <v>174</v>
+        <v>291</v>
       </c>
       <c r="F198" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G198" s="2" t="s">
-        <v>287</v>
+        <v>256</v>
       </c>
       <c r="H198" s="2" t="s">
-        <v>290</v>
+        <v>259</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4186,7 +4184,7 @@
       <c r="E199" s="4"/>
       <c r="F199" s="4"/>
       <c r="G199" s="2" t="s">
-        <v>288</v>
+        <v>257</v>
       </c>
       <c r="H199" s="1"/>
     </row>
@@ -4198,7 +4196,7 @@
       <c r="E200" s="4"/>
       <c r="F200" s="4"/>
       <c r="G200" s="2" t="s">
-        <v>289</v>
+        <v>258</v>
       </c>
       <c r="H200" s="1"/>
     </row>
@@ -4210,12 +4208,13 @@
       <c r="E201" s="5"/>
       <c r="F201" s="5"/>
       <c r="G201" s="2" t="s">
-        <v>282</v>
+        <v>251</v>
       </c>
       <c r="H201" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="300">
+    <mergeCell ref="C34:C37"/>
     <mergeCell ref="A114:A117"/>
     <mergeCell ref="E110:E113"/>
     <mergeCell ref="B38:B41"/>
@@ -4225,34 +4224,14 @@
     <mergeCell ref="C98:C101"/>
     <mergeCell ref="C154:C157"/>
     <mergeCell ref="E14:E17"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="E102:E105"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="A162:A165"/>
-    <mergeCell ref="C162:C165"/>
-    <mergeCell ref="B130:B133"/>
-    <mergeCell ref="E38:E41"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="E158:E161"/>
     <mergeCell ref="A18:A21"/>
     <mergeCell ref="D26:D29"/>
-    <mergeCell ref="B30:B33"/>
     <mergeCell ref="D14:D17"/>
-    <mergeCell ref="A158:A161"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="B154:B157"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="E62:E65"/>
-    <mergeCell ref="F50:F53"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="D46:D49"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="D198:D201"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="C58:C61"/>
     <mergeCell ref="F198:F201"/>
     <mergeCell ref="C146:C149"/>
     <mergeCell ref="D174:D177"/>
@@ -4269,11 +4248,15 @@
     <mergeCell ref="F98:F101"/>
     <mergeCell ref="C86:C89"/>
     <mergeCell ref="F82:F85"/>
-    <mergeCell ref="E130:E133"/>
-    <mergeCell ref="D54:D57"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="C138:C141"/>
-    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="E102:E105"/>
+    <mergeCell ref="A162:A165"/>
+    <mergeCell ref="C162:C165"/>
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="E158:E161"/>
+    <mergeCell ref="A158:A161"/>
+    <mergeCell ref="B154:B157"/>
+    <mergeCell ref="F190:F193"/>
     <mergeCell ref="F150:F153"/>
     <mergeCell ref="D150:D153"/>
     <mergeCell ref="A2:A5"/>
@@ -4297,10 +4280,6 @@
     <mergeCell ref="C102:C105"/>
     <mergeCell ref="A34:A37"/>
     <mergeCell ref="B26:B29"/>
-    <mergeCell ref="E50:E53"/>
-    <mergeCell ref="D82:D85"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="B194:B197"/>
     <mergeCell ref="D10:D13"/>
     <mergeCell ref="B90:B93"/>
     <mergeCell ref="D50:D53"/>
@@ -4312,7 +4291,6 @@
     <mergeCell ref="D178:D181"/>
     <mergeCell ref="D34:D37"/>
     <mergeCell ref="F178:F181"/>
-    <mergeCell ref="A182:A185"/>
     <mergeCell ref="C42:C45"/>
     <mergeCell ref="F34:F37"/>
     <mergeCell ref="F74:F77"/>
@@ -4320,10 +4298,12 @@
     <mergeCell ref="E42:E45"/>
     <mergeCell ref="B18:B21"/>
     <mergeCell ref="B106:B109"/>
-    <mergeCell ref="E186:E189"/>
-    <mergeCell ref="A194:A197"/>
     <mergeCell ref="C46:C49"/>
-    <mergeCell ref="F190:F193"/>
+    <mergeCell ref="E50:E53"/>
+    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="D46:D49"/>
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="D2:D5"/>
     <mergeCell ref="B42:B45"/>
@@ -4348,13 +4328,6 @@
     <mergeCell ref="E70:E73"/>
     <mergeCell ref="C106:C109"/>
     <mergeCell ref="A46:A49"/>
-    <mergeCell ref="C178:C181"/>
-    <mergeCell ref="E54:E57"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="D118:D121"/>
-    <mergeCell ref="F62:F65"/>
     <mergeCell ref="B198:B201"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="E198:E201"/>
@@ -4367,11 +4340,18 @@
     <mergeCell ref="D158:D161"/>
     <mergeCell ref="B98:B101"/>
     <mergeCell ref="A66:A69"/>
-    <mergeCell ref="F114:F117"/>
     <mergeCell ref="D154:D157"/>
     <mergeCell ref="A118:A121"/>
     <mergeCell ref="C118:C121"/>
-    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="A182:A185"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="A194:A197"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="D198:D201"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="B50:B53"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="C50:C53"/>
     <mergeCell ref="B82:B85"/>
@@ -4396,10 +4376,6 @@
     <mergeCell ref="A82:A85"/>
     <mergeCell ref="B110:B113"/>
     <mergeCell ref="E106:E109"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="B162:B165"/>
-    <mergeCell ref="A134:A137"/>
     <mergeCell ref="C194:C197"/>
     <mergeCell ref="C38:C41"/>
     <mergeCell ref="D58:D61"/>
@@ -4413,15 +4389,17 @@
     <mergeCell ref="C186:C189"/>
     <mergeCell ref="D94:D97"/>
     <mergeCell ref="E142:E145"/>
-    <mergeCell ref="C18:C21"/>
     <mergeCell ref="E194:E197"/>
     <mergeCell ref="B150:B153"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="D186:D189"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="F166:F169"/>
+    <mergeCell ref="A170:A173"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C170:C173"/>
+    <mergeCell ref="C178:C181"/>
+    <mergeCell ref="E54:E57"/>
+    <mergeCell ref="E178:E181"/>
     <mergeCell ref="B190:B193"/>
     <mergeCell ref="C26:C29"/>
     <mergeCell ref="D138:D141"/>
@@ -4441,23 +4419,35 @@
     <mergeCell ref="F182:F185"/>
     <mergeCell ref="D110:D113"/>
     <mergeCell ref="B54:B57"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="F166:F169"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C170:C173"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="F118:F121"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="B162:B165"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="D62:D65"/>
     <mergeCell ref="A110:A113"/>
     <mergeCell ref="E126:E129"/>
     <mergeCell ref="C166:C169"/>
     <mergeCell ref="B94:B97"/>
-    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="D186:D189"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="D118:D121"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="F114:F117"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="E38:E41"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="E130:E133"/>
+    <mergeCell ref="D54:D57"/>
+    <mergeCell ref="B134:B137"/>
     <mergeCell ref="F46:F49"/>
     <mergeCell ref="B166:B169"/>
     <mergeCell ref="E74:E77"/>
@@ -4468,6 +4458,14 @@
     <mergeCell ref="F94:F97"/>
     <mergeCell ref="B158:B161"/>
     <mergeCell ref="D78:D81"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="F118:F121"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="C138:C141"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="D82:D85"/>
     <mergeCell ref="D6:D9"/>
     <mergeCell ref="D190:D193"/>
     <mergeCell ref="B86:B89"/>

</xml_diff>